<commit_message>
Atualiza dashboards Aura - 2026-09-12 14:40:14
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -30767,7 +30767,7 @@
       </c>
       <c r="B490" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C490" s="2" t="inlineStr">
@@ -31821,7 +31821,7 @@
       </c>
       <c r="B507" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C507" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -38021,7 +38021,7 @@
       </c>
       <c r="B607" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C607" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51599,7 +51599,7 @@
       </c>
       <c r="B826" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C826" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -73609,7 +73609,7 @@
       </c>
       <c r="B1181" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1181" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77577,7 +77577,7 @@
       </c>
       <c r="B1245" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1245" s="2" t="inlineStr">
@@ -79375,7 +79375,7 @@
       </c>
       <c r="B1274" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1274" s="2" t="inlineStr">
@@ -79561,7 +79561,7 @@
       </c>
       <c r="B1277" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1277" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -92643,7 +92643,7 @@
       </c>
       <c r="B1488" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 14:50:18
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -31821,7 +31821,7 @@
       </c>
       <c r="B507" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C507" s="2" t="inlineStr">
@@ -33185,7 +33185,7 @@
       </c>
       <c r="B529" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C529" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="B612" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C612" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -42919,7 +42919,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -42981,7 +42981,7 @@
       </c>
       <c r="B687" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C687" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77577,7 +77577,7 @@
       </c>
       <c r="B1245" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1245" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83715,7 +83715,7 @@
       </c>
       <c r="B1344" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1344" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -88489,7 +88489,7 @@
       </c>
       <c r="B1421" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1421" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -92643,7 +92643,7 @@
       </c>
       <c r="B1488" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 15:00:21
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -31821,7 +31821,7 @@
       </c>
       <c r="B507" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C507" s="2" t="inlineStr">
@@ -33185,7 +33185,7 @@
       </c>
       <c r="B529" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C529" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -42981,7 +42981,7 @@
       </c>
       <c r="B687" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C687" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -79375,7 +79375,7 @@
       </c>
       <c r="B1274" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1274" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83715,7 +83715,7 @@
       </c>
       <c r="B1344" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1344" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84769,7 +84769,7 @@
       </c>
       <c r="B1361" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1361" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -88489,7 +88489,7 @@
       </c>
       <c r="B1421" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1421" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -91961,7 +91961,7 @@
       </c>
       <c r="B1477" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1477" s="2" t="inlineStr">
@@ -92643,7 +92643,7 @@
       </c>
       <c r="B1488" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 15:10:48
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -33061,7 +33061,7 @@
       </c>
       <c r="B527" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C527" s="2" t="inlineStr">
@@ -38021,7 +38021,7 @@
       </c>
       <c r="B607" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C607" s="2" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="B681" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C681" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51103,7 +51103,7 @@
       </c>
       <c r="B818" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C818" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -58233,7 +58233,7 @@
       </c>
       <c r="B933" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C933" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77763,7 +77763,7 @@
       </c>
       <c r="B1248" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1248" s="2" t="inlineStr">
@@ -79375,7 +79375,7 @@
       </c>
       <c r="B1274" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1274" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -84087,7 +84087,7 @@
       </c>
       <c r="B1350" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1350" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84769,7 +84769,7 @@
       </c>
       <c r="B1361" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1361" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -92643,7 +92643,7 @@
       </c>
       <c r="B1488" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 15:20:20
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
@@ -34921,7 +34921,7 @@
       </c>
       <c r="B557" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C557" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -38021,7 +38021,7 @@
       </c>
       <c r="B607" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C607" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="B681" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C681" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51103,7 +51103,7 @@
       </c>
       <c r="B818" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C818" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -71749,7 +71749,7 @@
       </c>
       <c r="B1151" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1151" s="2" t="inlineStr">
@@ -73609,7 +73609,7 @@
       </c>
       <c r="B1181" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1181" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -77763,7 +77763,7 @@
       </c>
       <c r="B1248" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1248" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83715,7 +83715,7 @@
       </c>
       <c r="B1344" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1344" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84769,7 +84769,7 @@
       </c>
       <c r="B1361" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1361" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91961,7 +91961,7 @@
       </c>
       <c r="B1477" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1477" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 15:30:03
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -33061,7 +33061,7 @@
       </c>
       <c r="B527" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C527" s="2" t="inlineStr">
@@ -34921,7 +34921,7 @@
       </c>
       <c r="B557" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C557" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="B612" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C612" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51599,7 +51599,7 @@
       </c>
       <c r="B826" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C826" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -58233,7 +58233,7 @@
       </c>
       <c r="B933" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C933" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71749,7 +71749,7 @@
       </c>
       <c r="B1151" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1151" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -79561,7 +79561,7 @@
       </c>
       <c r="B1277" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1277" s="2" t="inlineStr">
@@ -79747,7 +79747,7 @@
       </c>
       <c r="B1280" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1280" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83715,7 +83715,7 @@
       </c>
       <c r="B1344" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1344" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84087,7 +84087,7 @@
       </c>
       <c r="B1350" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1350" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84769,7 +84769,7 @@
       </c>
       <c r="B1361" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1361" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -91961,7 +91961,7 @@
       </c>
       <c r="B1477" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1477" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 15:40:21
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -29713,7 +29713,7 @@
       </c>
       <c r="B473" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C473" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="B612" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C612" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -73609,7 +73609,7 @@
       </c>
       <c r="B1181" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1181" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -79561,7 +79561,7 @@
       </c>
       <c r="B1277" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1277" s="2" t="inlineStr">
@@ -79747,7 +79747,7 @@
       </c>
       <c r="B1280" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1280" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83715,7 +83715,7 @@
       </c>
       <c r="B1344" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1344" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84769,7 +84769,7 @@
       </c>
       <c r="B1361" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1361" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91961,7 +91961,7 @@
       </c>
       <c r="B1477" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1477" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 15:50:07
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -29713,7 +29713,7 @@
       </c>
       <c r="B473" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C473" s="2" t="inlineStr">
@@ -30767,7 +30767,7 @@
       </c>
       <c r="B490" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C490" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -33185,7 +33185,7 @@
       </c>
       <c r="B529" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C529" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="B612" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C612" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51599,7 +51599,7 @@
       </c>
       <c r="B826" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C826" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -73609,7 +73609,7 @@
       </c>
       <c r="B1181" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1181" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -79747,7 +79747,7 @@
       </c>
       <c r="B1280" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1280" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83715,7 +83715,7 @@
       </c>
       <c r="B1344" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1344" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -91961,7 +91961,7 @@
       </c>
       <c r="B1477" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1477" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 16:00:13
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -33185,7 +33185,7 @@
       </c>
       <c r="B529" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C529" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77577,7 +77577,7 @@
       </c>
       <c r="B1245" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1245" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -79375,7 +79375,7 @@
       </c>
       <c r="B1274" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1274" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84769,7 +84769,7 @@
       </c>
       <c r="B1361" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1361" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91031,7 +91031,7 @@
       </c>
       <c r="B1462" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1462" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 16:10:52
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -30767,7 +30767,7 @@
       </c>
       <c r="B490" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C490" s="2" t="inlineStr">
@@ -31821,7 +31821,7 @@
       </c>
       <c r="B507" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C507" s="2" t="inlineStr">
@@ -34921,7 +34921,7 @@
       </c>
       <c r="B557" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C557" s="2" t="inlineStr">
@@ -35541,7 +35541,7 @@
       </c>
       <c r="B567" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C567" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="B612" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C612" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="B681" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C681" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -60279,7 +60279,7 @@
       </c>
       <c r="B966" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C966" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71749,7 +71749,7 @@
       </c>
       <c r="B1151" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1151" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -74973,7 +74973,7 @@
       </c>
       <c r="B1203" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1203" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77577,7 +77577,7 @@
       </c>
       <c r="B1245" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1245" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -79375,7 +79375,7 @@
       </c>
       <c r="B1274" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1274" s="2" t="inlineStr">
@@ -79747,7 +79747,7 @@
       </c>
       <c r="B1280" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1280" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84769,7 +84769,7 @@
       </c>
       <c r="B1361" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1361" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91031,7 +91031,7 @@
       </c>
       <c r="B1462" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1462" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -91961,7 +91961,7 @@
       </c>
       <c r="B1477" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1477" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 16:20:29
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -31821,7 +31821,7 @@
       </c>
       <c r="B507" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C507" s="2" t="inlineStr">
@@ -34921,7 +34921,7 @@
       </c>
       <c r="B557" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C557" s="2" t="inlineStr">
@@ -35541,7 +35541,7 @@
       </c>
       <c r="B567" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C567" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="B681" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C681" s="2" t="inlineStr">
@@ -42919,7 +42919,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -42981,7 +42981,7 @@
       </c>
       <c r="B687" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C687" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -60279,7 +60279,7 @@
       </c>
       <c r="B966" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C966" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -71749,7 +71749,7 @@
       </c>
       <c r="B1151" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1151" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -74973,7 +74973,7 @@
       </c>
       <c r="B1203" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1203" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -79561,7 +79561,7 @@
       </c>
       <c r="B1277" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1277" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84769,7 +84769,7 @@
       </c>
       <c r="B1361" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1361" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -86629,7 +86629,7 @@
       </c>
       <c r="B1391" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1391" s="2" t="inlineStr">
@@ -88489,7 +88489,7 @@
       </c>
       <c r="B1421" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1421" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 16:30:14
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -35541,7 +35541,7 @@
       </c>
       <c r="B567" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C567" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="B681" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C681" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -42919,7 +42919,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -42981,7 +42981,7 @@
       </c>
       <c r="B687" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C687" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -58233,7 +58233,7 @@
       </c>
       <c r="B933" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C933" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -74601,7 +74601,7 @@
       </c>
       <c r="B1197" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1197" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -77763,7 +77763,7 @@
       </c>
       <c r="B1248" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1248" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -79561,7 +79561,7 @@
       </c>
       <c r="B1277" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1277" s="2" t="inlineStr">
@@ -79747,7 +79747,7 @@
       </c>
       <c r="B1280" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1280" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -84087,7 +84087,7 @@
       </c>
       <c r="B1350" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1350" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -86629,7 +86629,7 @@
       </c>
       <c r="B1391" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1391" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -88489,7 +88489,7 @@
       </c>
       <c r="B1421" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1421" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -92643,7 +92643,7 @@
       </c>
       <c r="B1488" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 16:40:21
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -31821,7 +31821,7 @@
       </c>
       <c r="B507" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C507" s="2" t="inlineStr">
@@ -35541,7 +35541,7 @@
       </c>
       <c r="B567" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C567" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="B681" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C681" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51599,7 +51599,7 @@
       </c>
       <c r="B826" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C826" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -58233,7 +58233,7 @@
       </c>
       <c r="B933" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C933" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -77763,7 +77763,7 @@
       </c>
       <c r="B1248" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1248" s="2" t="inlineStr">
@@ -79747,7 +79747,7 @@
       </c>
       <c r="B1280" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1280" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -84087,7 +84087,7 @@
       </c>
       <c r="B1350" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1350" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84769,7 +84769,7 @@
       </c>
       <c r="B1361" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1361" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -91961,7 +91961,7 @@
       </c>
       <c r="B1477" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1477" s="2" t="inlineStr">
@@ -92643,7 +92643,7 @@
       </c>
       <c r="B1488" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 16:50:29
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -30767,7 +30767,7 @@
       </c>
       <c r="B490" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C490" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="B612" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C612" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -42919,7 +42919,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -42981,7 +42981,7 @@
       </c>
       <c r="B687" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C687" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51599,7 +51599,7 @@
       </c>
       <c r="B826" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C826" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -58233,7 +58233,7 @@
       </c>
       <c r="B933" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C933" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -74601,7 +74601,7 @@
       </c>
       <c r="B1197" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1197" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -74973,7 +74973,7 @@
       </c>
       <c r="B1203" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1203" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77763,7 +77763,7 @@
       </c>
       <c r="B1248" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1248" s="2" t="inlineStr">
@@ -79561,7 +79561,7 @@
       </c>
       <c r="B1277" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1277" s="2" t="inlineStr">
@@ -79747,7 +79747,7 @@
       </c>
       <c r="B1280" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1280" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 17:00:37
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -30767,7 +30767,7 @@
       </c>
       <c r="B490" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C490" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="B681" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C681" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -42919,7 +42919,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -42981,7 +42981,7 @@
       </c>
       <c r="B687" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C687" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -58233,7 +58233,7 @@
       </c>
       <c r="B933" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C933" s="2" t="inlineStr">
@@ -60279,7 +60279,7 @@
       </c>
       <c r="B966" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C966" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -73609,7 +73609,7 @@
       </c>
       <c r="B1181" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1181" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -74973,7 +74973,7 @@
       </c>
       <c r="B1203" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1203" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77763,7 +77763,7 @@
       </c>
       <c r="B1248" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1248" s="2" t="inlineStr">
@@ -79561,7 +79561,7 @@
       </c>
       <c r="B1277" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1277" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84769,7 +84769,7 @@
       </c>
       <c r="B1361" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1361" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -86629,7 +86629,7 @@
       </c>
       <c r="B1391" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1391" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -88489,7 +88489,7 @@
       </c>
       <c r="B1421" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1421" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 17:10:49
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -31821,7 +31821,7 @@
       </c>
       <c r="B507" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C507" s="2" t="inlineStr">
@@ -35541,7 +35541,7 @@
       </c>
       <c r="B567" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C567" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -51103,7 +51103,7 @@
       </c>
       <c r="B818" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C818" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -60279,7 +60279,7 @@
       </c>
       <c r="B966" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C966" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -79747,7 +79747,7 @@
       </c>
       <c r="B1280" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1280" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84769,7 +84769,7 @@
       </c>
       <c r="B1361" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1361" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -86629,7 +86629,7 @@
       </c>
       <c r="B1391" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1391" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 17:20:14
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -30767,7 +30767,7 @@
       </c>
       <c r="B490" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C490" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
@@ -34921,7 +34921,7 @@
       </c>
       <c r="B557" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C557" s="2" t="inlineStr">
@@ -35541,7 +35541,7 @@
       </c>
       <c r="B567" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C567" s="2" t="inlineStr">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="B612" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C612" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -42919,7 +42919,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51103,7 +51103,7 @@
       </c>
       <c r="B818" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C818" s="2" t="inlineStr">
@@ -51599,7 +51599,7 @@
       </c>
       <c r="B826" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C826" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -73609,7 +73609,7 @@
       </c>
       <c r="B1181" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1181" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -88489,7 +88489,7 @@
       </c>
       <c r="B1421" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1421" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91031,7 +91031,7 @@
       </c>
       <c r="B1462" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1462" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 17:30:10
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -30767,7 +30767,7 @@
       </c>
       <c r="B490" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C490" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
@@ -33185,7 +33185,7 @@
       </c>
       <c r="B529" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C529" s="2" t="inlineStr">
@@ -34921,7 +34921,7 @@
       </c>
       <c r="B557" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C557" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="B681" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C681" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -42919,7 +42919,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51103,7 +51103,7 @@
       </c>
       <c r="B818" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C818" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51599,7 +51599,7 @@
       </c>
       <c r="B826" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C826" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -60279,7 +60279,7 @@
       </c>
       <c r="B966" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C966" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77577,7 +77577,7 @@
       </c>
       <c r="B1245" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1245" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -79747,7 +79747,7 @@
       </c>
       <c r="B1280" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1280" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84769,7 +84769,7 @@
       </c>
       <c r="B1361" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1361" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -88489,7 +88489,7 @@
       </c>
       <c r="B1421" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1421" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -91031,7 +91031,7 @@
       </c>
       <c r="B1462" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1462" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -92643,7 +92643,7 @@
       </c>
       <c r="B1488" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 17:40:50
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -30767,7 +30767,7 @@
       </c>
       <c r="B490" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C490" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -42919,7 +42919,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51103,7 +51103,7 @@
       </c>
       <c r="B818" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C818" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51599,7 +51599,7 @@
       </c>
       <c r="B826" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C826" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -60279,7 +60279,7 @@
       </c>
       <c r="B966" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C966" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -73609,7 +73609,7 @@
       </c>
       <c r="B1181" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1181" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77577,7 +77577,7 @@
       </c>
       <c r="B1245" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1245" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -79561,7 +79561,7 @@
       </c>
       <c r="B1277" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1277" s="2" t="inlineStr">
@@ -79747,7 +79747,7 @@
       </c>
       <c r="B1280" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1280" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -88489,7 +88489,7 @@
       </c>
       <c r="B1421" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1421" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -92643,7 +92643,7 @@
       </c>
       <c r="B1488" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 17:52:48
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -30767,7 +30767,7 @@
       </c>
       <c r="B490" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C490" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -33185,7 +33185,7 @@
       </c>
       <c r="B529" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C529" s="2" t="inlineStr">
@@ -35541,7 +35541,7 @@
       </c>
       <c r="B567" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C567" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42919,7 +42919,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -79747,7 +79747,7 @@
       </c>
       <c r="B1280" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1280" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -92643,7 +92643,7 @@
       </c>
       <c r="B1488" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 18:01:39
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -38021,7 +38021,7 @@
       </c>
       <c r="B607" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C607" s="2" t="inlineStr">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="B612" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C612" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -42981,7 +42981,7 @@
       </c>
       <c r="B687" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C687" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -58233,7 +58233,7 @@
       </c>
       <c r="B933" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C933" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77763,7 +77763,7 @@
       </c>
       <c r="B1248" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1248" s="2" t="inlineStr">
@@ -79561,7 +79561,7 @@
       </c>
       <c r="B1277" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1277" s="2" t="inlineStr">
@@ -79747,7 +79747,7 @@
       </c>
       <c r="B1280" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1280" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84087,7 +84087,7 @@
       </c>
       <c r="B1350" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1350" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -86629,7 +86629,7 @@
       </c>
       <c r="B1391" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1391" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91031,7 +91031,7 @@
       </c>
       <c r="B1462" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1462" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -91961,7 +91961,7 @@
       </c>
       <c r="B1477" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1477" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 18:11:45
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
@@ -35541,7 +35541,7 @@
       </c>
       <c r="B567" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C567" s="2" t="inlineStr">
@@ -38021,7 +38021,7 @@
       </c>
       <c r="B607" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C607" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="B681" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C681" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -42981,7 +42981,7 @@
       </c>
       <c r="B687" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C687" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -51599,7 +51599,7 @@
       </c>
       <c r="B826" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C826" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -58233,7 +58233,7 @@
       </c>
       <c r="B933" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C933" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -77763,7 +77763,7 @@
       </c>
       <c r="B1248" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1248" s="2" t="inlineStr">
@@ -79561,7 +79561,7 @@
       </c>
       <c r="B1277" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1277" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -86629,7 +86629,7 @@
       </c>
       <c r="B1391" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1391" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -88489,7 +88489,7 @@
       </c>
       <c r="B1421" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1421" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -91031,7 +91031,7 @@
       </c>
       <c r="B1462" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1462" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -92643,7 +92643,7 @@
       </c>
       <c r="B1488" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 18:21:51
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -35541,7 +35541,7 @@
       </c>
       <c r="B567" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C567" s="2" t="inlineStr">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="B612" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C612" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="B681" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C681" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -42919,7 +42919,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -73609,7 +73609,7 @@
       </c>
       <c r="B1181" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1181" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -77763,7 +77763,7 @@
       </c>
       <c r="B1248" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1248" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -84087,7 +84087,7 @@
       </c>
       <c r="B1350" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1350" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -88489,7 +88489,7 @@
       </c>
       <c r="B1421" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1421" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -91031,7 +91031,7 @@
       </c>
       <c r="B1462" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1462" s="2" t="inlineStr">
@@ -91961,7 +91961,7 @@
       </c>
       <c r="B1477" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1477" s="2" t="inlineStr">
@@ -92643,7 +92643,7 @@
       </c>
       <c r="B1488" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 18:33:25
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
@@ -34921,7 +34921,7 @@
       </c>
       <c r="B557" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C557" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="B612" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C612" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="B681" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C681" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -42919,7 +42919,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -51103,7 +51103,7 @@
       </c>
       <c r="B818" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C818" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -58233,7 +58233,7 @@
       </c>
       <c r="B933" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C933" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77577,7 +77577,7 @@
       </c>
       <c r="B1245" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1245" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -79561,7 +79561,7 @@
       </c>
       <c r="B1277" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1277" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84087,7 +84087,7 @@
       </c>
       <c r="B1350" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1350" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91031,7 +91031,7 @@
       </c>
       <c r="B1462" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1462" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -91961,7 +91961,7 @@
       </c>
       <c r="B1477" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1477" s="2" t="inlineStr">
@@ -92643,7 +92643,7 @@
       </c>
       <c r="B1488" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 18:42:50
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -34921,7 +34921,7 @@
       </c>
       <c r="B557" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C557" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -42981,7 +42981,7 @@
       </c>
       <c r="B687" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C687" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51103,7 +51103,7 @@
       </c>
       <c r="B818" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C818" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -58233,7 +58233,7 @@
       </c>
       <c r="B933" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C933" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -73609,7 +73609,7 @@
       </c>
       <c r="B1181" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1181" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77577,7 +77577,7 @@
       </c>
       <c r="B1245" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1245" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -77763,7 +77763,7 @@
       </c>
       <c r="B1248" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1248" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -79561,7 +79561,7 @@
       </c>
       <c r="B1277" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1277" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -84087,7 +84087,7 @@
       </c>
       <c r="B1350" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1350" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 18:53:13
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -29713,7 +29713,7 @@
       </c>
       <c r="B473" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C473" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -38021,7 +38021,7 @@
       </c>
       <c r="B607" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C607" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="B681" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C681" s="2" t="inlineStr">
@@ -42919,7 +42919,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -42981,7 +42981,7 @@
       </c>
       <c r="B687" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C687" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51103,7 +51103,7 @@
       </c>
       <c r="B818" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C818" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -73609,7 +73609,7 @@
       </c>
       <c r="B1181" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1181" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -79375,7 +79375,7 @@
       </c>
       <c r="B1274" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1274" s="2" t="inlineStr">
@@ -79561,7 +79561,7 @@
       </c>
       <c r="B1277" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1277" s="2" t="inlineStr">
@@ -79747,7 +79747,7 @@
       </c>
       <c r="B1280" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1280" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -84087,7 +84087,7 @@
       </c>
       <c r="B1350" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1350" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 19:02:28
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -29713,7 +29713,7 @@
       </c>
       <c r="B473" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C473" s="2" t="inlineStr">
@@ -30767,7 +30767,7 @@
       </c>
       <c r="B490" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C490" s="2" t="inlineStr">
@@ -35541,7 +35541,7 @@
       </c>
       <c r="B567" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C567" s="2" t="inlineStr">
@@ -38021,7 +38021,7 @@
       </c>
       <c r="B607" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C607" s="2" t="inlineStr">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="B612" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C612" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -42919,7 +42919,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -42981,7 +42981,7 @@
       </c>
       <c r="B687" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C687" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51103,7 +51103,7 @@
       </c>
       <c r="B818" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C818" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51599,7 +51599,7 @@
       </c>
       <c r="B826" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C826" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -73609,7 +73609,7 @@
       </c>
       <c r="B1181" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1181" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -79375,7 +79375,7 @@
       </c>
       <c r="B1274" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1274" s="2" t="inlineStr">
@@ -79747,7 +79747,7 @@
       </c>
       <c r="B1280" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1280" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84087,7 +84087,7 @@
       </c>
       <c r="B1350" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1350" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -91961,7 +91961,7 @@
       </c>
       <c r="B1477" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1477" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 19:13:00
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -29713,7 +29713,7 @@
       </c>
       <c r="B473" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C473" s="2" t="inlineStr">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="B612" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C612" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51103,7 +51103,7 @@
       </c>
       <c r="B818" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C818" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -58233,7 +58233,7 @@
       </c>
       <c r="B933" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C933" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -79747,7 +79747,7 @@
       </c>
       <c r="B1280" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1280" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -86629,7 +86629,7 @@
       </c>
       <c r="B1391" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1391" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 19:22:37
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -29713,7 +29713,7 @@
       </c>
       <c r="B473" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C473" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
@@ -33061,7 +33061,7 @@
       </c>
       <c r="B527" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C527" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51103,7 +51103,7 @@
       </c>
       <c r="B818" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C818" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51599,7 +51599,7 @@
       </c>
       <c r="B826" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C826" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -60279,7 +60279,7 @@
       </c>
       <c r="B966" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C966" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -77763,7 +77763,7 @@
       </c>
       <c r="B1248" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1248" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -79375,7 +79375,7 @@
       </c>
       <c r="B1274" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1274" s="2" t="inlineStr">
@@ -79561,7 +79561,7 @@
       </c>
       <c r="B1277" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1277" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83715,7 +83715,7 @@
       </c>
       <c r="B1344" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1344" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -86629,7 +86629,7 @@
       </c>
       <c r="B1391" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1391" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -92643,7 +92643,7 @@
       </c>
       <c r="B1488" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 19:33:34
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -58233,7 +58233,7 @@
       </c>
       <c r="B933" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C933" s="2" t="inlineStr">
@@ -60279,7 +60279,7 @@
       </c>
       <c r="B966" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C966" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71749,7 +71749,7 @@
       </c>
       <c r="B1151" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1151" s="2" t="inlineStr">
@@ -73609,7 +73609,7 @@
       </c>
       <c r="B1181" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1181" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -74973,7 +74973,7 @@
       </c>
       <c r="B1203" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1203" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -79375,7 +79375,7 @@
       </c>
       <c r="B1274" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1274" s="2" t="inlineStr">
@@ -79561,7 +79561,7 @@
       </c>
       <c r="B1277" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1277" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83715,7 +83715,7 @@
       </c>
       <c r="B1344" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1344" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 19:43:16
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -30767,7 +30767,7 @@
       </c>
       <c r="B490" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C490" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
@@ -33061,7 +33061,7 @@
       </c>
       <c r="B527" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C527" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -42981,7 +42981,7 @@
       </c>
       <c r="B687" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C687" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51103,7 +51103,7 @@
       </c>
       <c r="B818" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C818" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -74601,7 +74601,7 @@
       </c>
       <c r="B1197" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1197" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -74973,7 +74973,7 @@
       </c>
       <c r="B1203" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1203" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -77763,7 +77763,7 @@
       </c>
       <c r="B1248" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1248" s="2" t="inlineStr">
@@ -79561,7 +79561,7 @@
       </c>
       <c r="B1277" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1277" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -86629,7 +86629,7 @@
       </c>
       <c r="B1391" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1391" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -91961,7 +91961,7 @@
       </c>
       <c r="B1477" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1477" s="2" t="inlineStr">
@@ -92643,7 +92643,7 @@
       </c>
       <c r="B1488" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 19:53:11
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -71749,7 +71749,7 @@
       </c>
       <c r="B1151" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1151" s="2" t="inlineStr">
@@ -73609,7 +73609,7 @@
       </c>
       <c r="B1181" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1181" s="2" t="inlineStr">
@@ -74601,7 +74601,7 @@
       </c>
       <c r="B1197" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1197" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84769,7 +84769,7 @@
       </c>
       <c r="B1361" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1361" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -86629,7 +86629,7 @@
       </c>
       <c r="B1391" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1391" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -91961,7 +91961,7 @@
       </c>
       <c r="B1477" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1477" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 20:03:41
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51103,7 +51103,7 @@
       </c>
       <c r="B818" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C818" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -58233,7 +58233,7 @@
       </c>
       <c r="B933" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C933" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -73609,7 +73609,7 @@
       </c>
       <c r="B1181" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1181" s="2" t="inlineStr">
@@ -74601,7 +74601,7 @@
       </c>
       <c r="B1197" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1197" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -77577,7 +77577,7 @@
       </c>
       <c r="B1245" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1245" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -79375,7 +79375,7 @@
       </c>
       <c r="B1274" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1274" s="2" t="inlineStr">
@@ -79561,7 +79561,7 @@
       </c>
       <c r="B1277" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1277" s="2" t="inlineStr">
@@ -79747,7 +79747,7 @@
       </c>
       <c r="B1280" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1280" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 20:16:18
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -34921,7 +34921,7 @@
       </c>
       <c r="B557" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C557" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -42981,7 +42981,7 @@
       </c>
       <c r="B687" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C687" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -58233,7 +58233,7 @@
       </c>
       <c r="B933" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C933" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -74601,7 +74601,7 @@
       </c>
       <c r="B1197" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1197" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -74973,7 +74973,7 @@
       </c>
       <c r="B1203" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1203" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -79375,7 +79375,7 @@
       </c>
       <c r="B1274" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1274" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84769,7 +84769,7 @@
       </c>
       <c r="B1361" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1361" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -88489,7 +88489,7 @@
       </c>
       <c r="B1421" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1421" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -91961,7 +91961,7 @@
       </c>
       <c r="B1477" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1477" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 20:25:14
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -29713,7 +29713,7 @@
       </c>
       <c r="B473" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C473" s="2" t="inlineStr">
@@ -31821,7 +31821,7 @@
       </c>
       <c r="B507" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C507" s="2" t="inlineStr">
@@ -34425,7 +34425,7 @@
       </c>
       <c r="B549" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C549" s="2" t="inlineStr">
@@ -34921,7 +34921,7 @@
       </c>
       <c r="B557" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C557" s="2" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="B681" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C681" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -42981,7 +42981,7 @@
       </c>
       <c r="B687" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C687" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -74601,7 +74601,7 @@
       </c>
       <c r="B1197" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1197" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -74973,7 +74973,7 @@
       </c>
       <c r="B1203" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1203" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -77577,7 +77577,7 @@
       </c>
       <c r="B1245" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1245" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -88489,7 +88489,7 @@
       </c>
       <c r="B1421" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1421" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91031,7 +91031,7 @@
       </c>
       <c r="B1462" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1462" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 20:35:20
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -29713,7 +29713,7 @@
       </c>
       <c r="B473" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C473" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
@@ -33185,7 +33185,7 @@
       </c>
       <c r="B529" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C529" s="2" t="inlineStr">
@@ -34425,7 +34425,7 @@
       </c>
       <c r="B549" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C549" s="2" t="inlineStr">
@@ -35541,7 +35541,7 @@
       </c>
       <c r="B567" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C567" s="2" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="B681" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C681" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -74601,7 +74601,7 @@
       </c>
       <c r="B1197" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1197" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -79561,7 +79561,7 @@
       </c>
       <c r="B1277" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1277" s="2" t="inlineStr">
@@ -79747,7 +79747,7 @@
       </c>
       <c r="B1280" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1280" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -91031,7 +91031,7 @@
       </c>
       <c r="B1462" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1462" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 20:45:28
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -30767,7 +30767,7 @@
       </c>
       <c r="B490" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C490" s="2" t="inlineStr">
@@ -31821,7 +31821,7 @@
       </c>
       <c r="B507" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C507" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
@@ -33061,7 +33061,7 @@
       </c>
       <c r="B527" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C527" s="2" t="inlineStr">
@@ -33185,7 +33185,7 @@
       </c>
       <c r="B529" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C529" s="2" t="inlineStr">
@@ -34425,7 +34425,7 @@
       </c>
       <c r="B549" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C549" s="2" t="inlineStr">
@@ -35541,7 +35541,7 @@
       </c>
       <c r="B567" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C567" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="B612" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C612" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -42981,7 +42981,7 @@
       </c>
       <c r="B687" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C687" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77577,7 +77577,7 @@
       </c>
       <c r="B1245" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1245" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 20:59:40
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -33061,7 +33061,7 @@
       </c>
       <c r="B527" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C527" s="2" t="inlineStr">
@@ -34425,7 +34425,7 @@
       </c>
       <c r="B549" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C549" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="B612" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C612" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="B681" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C681" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -58233,7 +58233,7 @@
       </c>
       <c r="B933" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C933" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -77577,7 +77577,7 @@
       </c>
       <c r="B1245" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1245" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -79561,7 +79561,7 @@
       </c>
       <c r="B1277" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1277" s="2" t="inlineStr">
@@ -79747,7 +79747,7 @@
       </c>
       <c r="B1280" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1280" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -86629,7 +86629,7 @@
       </c>
       <c r="B1391" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1391" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -91961,7 +91961,7 @@
       </c>
       <c r="B1477" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1477" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 21:11:24
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -30767,7 +30767,7 @@
       </c>
       <c r="B490" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C490" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -31821,7 +31821,7 @@
       </c>
       <c r="B507" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C507" s="2" t="inlineStr">
@@ -35541,7 +35541,7 @@
       </c>
       <c r="B567" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C567" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -42919,7 +42919,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -58233,7 +58233,7 @@
       </c>
       <c r="B933" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C933" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -86629,7 +86629,7 @@
       </c>
       <c r="B1391" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1391" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -91031,7 +91031,7 @@
       </c>
       <c r="B1462" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1462" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 21:23:42
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -31821,7 +31821,7 @@
       </c>
       <c r="B507" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C507" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
@@ -33061,7 +33061,7 @@
       </c>
       <c r="B527" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C527" s="2" t="inlineStr">
@@ -35541,7 +35541,7 @@
       </c>
       <c r="B567" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C567" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="B681" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C681" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -42919,7 +42919,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -42981,7 +42981,7 @@
       </c>
       <c r="B687" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C687" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71749,7 +71749,7 @@
       </c>
       <c r="B1151" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1151" s="2" t="inlineStr">
@@ -73609,7 +73609,7 @@
       </c>
       <c r="B1181" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1181" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -91031,7 +91031,7 @@
       </c>
       <c r="B1462" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1462" s="2" t="inlineStr">
@@ -91961,7 +91961,7 @@
       </c>
       <c r="B1477" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1477" s="2" t="inlineStr">
@@ -92643,7 +92643,7 @@
       </c>
       <c r="B1488" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 21:37:19
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -29713,7 +29713,7 @@
       </c>
       <c r="B473" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C473" s="2" t="inlineStr">
@@ -30767,7 +30767,7 @@
       </c>
       <c r="B490" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C490" s="2" t="inlineStr">
@@ -31821,7 +31821,7 @@
       </c>
       <c r="B507" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C507" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
@@ -33061,7 +33061,7 @@
       </c>
       <c r="B527" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C527" s="2" t="inlineStr">
@@ -34921,7 +34921,7 @@
       </c>
       <c r="B557" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C557" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -38021,7 +38021,7 @@
       </c>
       <c r="B607" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C607" s="2" t="inlineStr">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="B612" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C612" s="2" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="B681" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C681" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71749,7 +71749,7 @@
       </c>
       <c r="B1151" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1151" s="2" t="inlineStr">
@@ -74601,7 +74601,7 @@
       </c>
       <c r="B1197" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1197" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -77577,7 +77577,7 @@
       </c>
       <c r="B1245" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1245" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -77763,7 +77763,7 @@
       </c>
       <c r="B1248" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1248" s="2" t="inlineStr">
@@ -83715,7 +83715,7 @@
       </c>
       <c r="B1344" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1344" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -91961,7 +91961,7 @@
       </c>
       <c r="B1477" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1477" s="2" t="inlineStr">
@@ -92643,7 +92643,7 @@
       </c>
       <c r="B1488" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 21:48:49
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -31821,7 +31821,7 @@
       </c>
       <c r="B507" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C507" s="2" t="inlineStr">
@@ -34921,7 +34921,7 @@
       </c>
       <c r="B557" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C557" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -38021,7 +38021,7 @@
       </c>
       <c r="B607" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C607" s="2" t="inlineStr">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="B612" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C612" s="2" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="B681" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C681" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -74601,7 +74601,7 @@
       </c>
       <c r="B1197" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1197" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77577,7 +77577,7 @@
       </c>
       <c r="B1245" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1245" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -77763,7 +77763,7 @@
       </c>
       <c r="B1248" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1248" s="2" t="inlineStr">
@@ -79747,7 +79747,7 @@
       </c>
       <c r="B1280" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1280" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83715,7 +83715,7 @@
       </c>
       <c r="B1344" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1344" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84769,7 +84769,7 @@
       </c>
       <c r="B1361" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1361" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91031,7 +91031,7 @@
       </c>
       <c r="B1462" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1462" s="2" t="inlineStr">
@@ -91961,7 +91961,7 @@
       </c>
       <c r="B1477" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1477" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 22:01:11
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -30767,7 +30767,7 @@
       </c>
       <c r="B490" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C490" s="2" t="inlineStr">
@@ -31821,7 +31821,7 @@
       </c>
       <c r="B507" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C507" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -58233,7 +58233,7 @@
       </c>
       <c r="B933" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C933" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -73609,7 +73609,7 @@
       </c>
       <c r="B1181" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1181" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -74973,7 +74973,7 @@
       </c>
       <c r="B1203" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1203" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -79375,7 +79375,7 @@
       </c>
       <c r="B1274" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1274" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84769,7 +84769,7 @@
       </c>
       <c r="B1361" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1361" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -86629,7 +86629,7 @@
       </c>
       <c r="B1391" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1391" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -91031,7 +91031,7 @@
       </c>
       <c r="B1462" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1462" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -91961,7 +91961,7 @@
       </c>
       <c r="B1477" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1477" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 22:10:34
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -29713,7 +29713,7 @@
       </c>
       <c r="B473" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C473" s="2" t="inlineStr">
@@ -31821,7 +31821,7 @@
       </c>
       <c r="B507" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C507" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -74973,7 +74973,7 @@
       </c>
       <c r="B1203" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1203" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -79375,7 +79375,7 @@
       </c>
       <c r="B1274" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1274" s="2" t="inlineStr">
@@ -79561,7 +79561,7 @@
       </c>
       <c r="B1277" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1277" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -86629,7 +86629,7 @@
       </c>
       <c r="B1391" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1391" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -91961,7 +91961,7 @@
       </c>
       <c r="B1477" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1477" s="2" t="inlineStr">
@@ -92643,7 +92643,7 @@
       </c>
       <c r="B1488" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 22:20:08
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -30767,7 +30767,7 @@
       </c>
       <c r="B490" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C490" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -38021,7 +38021,7 @@
       </c>
       <c r="B607" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C607" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -42981,7 +42981,7 @@
       </c>
       <c r="B687" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C687" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51103,7 +51103,7 @@
       </c>
       <c r="B818" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C818" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -73609,7 +73609,7 @@
       </c>
       <c r="B1181" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1181" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74973,7 +74973,7 @@
       </c>
       <c r="B1203" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1203" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -77763,7 +77763,7 @@
       </c>
       <c r="B1248" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1248" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -91961,7 +91961,7 @@
       </c>
       <c r="B1477" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1477" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 22:30:06
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -30767,7 +30767,7 @@
       </c>
       <c r="B490" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C490" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -38021,7 +38021,7 @@
       </c>
       <c r="B607" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C607" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -42919,7 +42919,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -42981,7 +42981,7 @@
       </c>
       <c r="B687" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C687" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51103,7 +51103,7 @@
       </c>
       <c r="B818" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C818" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -73609,7 +73609,7 @@
       </c>
       <c r="B1181" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1181" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -74973,7 +74973,7 @@
       </c>
       <c r="B1203" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1203" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -77763,7 +77763,7 @@
       </c>
       <c r="B1248" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1248" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -84087,7 +84087,7 @@
       </c>
       <c r="B1350" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1350" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -88489,7 +88489,7 @@
       </c>
       <c r="B1421" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1421" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 22:41:16
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -34425,7 +34425,7 @@
       </c>
       <c r="B549" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C549" s="2" t="inlineStr">
@@ -34921,7 +34921,7 @@
       </c>
       <c r="B557" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C557" s="2" t="inlineStr">
@@ -35541,7 +35541,7 @@
       </c>
       <c r="B567" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C567" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="B612" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C612" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="B681" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C681" s="2" t="inlineStr">
@@ -42919,7 +42919,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -42981,7 +42981,7 @@
       </c>
       <c r="B687" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C687" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51599,7 +51599,7 @@
       </c>
       <c r="B826" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C826" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -58233,7 +58233,7 @@
       </c>
       <c r="B933" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C933" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -79747,7 +79747,7 @@
       </c>
       <c r="B1280" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1280" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -84087,7 +84087,7 @@
       </c>
       <c r="B1350" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1350" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -86629,7 +86629,7 @@
       </c>
       <c r="B1391" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1391" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -92643,7 +92643,7 @@
       </c>
       <c r="B1488" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 22:50:30
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -31821,7 +31821,7 @@
       </c>
       <c r="B507" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C507" s="2" t="inlineStr">
@@ -34425,7 +34425,7 @@
       </c>
       <c r="B549" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C549" s="2" t="inlineStr">
@@ -34921,7 +34921,7 @@
       </c>
       <c r="B557" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C557" s="2" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="B681" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C681" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -58233,7 +58233,7 @@
       </c>
       <c r="B933" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C933" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -73609,7 +73609,7 @@
       </c>
       <c r="B1181" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1181" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -74973,7 +74973,7 @@
       </c>
       <c r="B1203" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1203" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77577,7 +77577,7 @@
       </c>
       <c r="B1245" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1245" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -79747,7 +79747,7 @@
       </c>
       <c r="B1280" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1280" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -92643,7 +92643,7 @@
       </c>
       <c r="B1488" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 23:01:09
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -31821,7 +31821,7 @@
       </c>
       <c r="B507" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C507" s="2" t="inlineStr">
@@ -34921,7 +34921,7 @@
       </c>
       <c r="B557" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C557" s="2" t="inlineStr">
@@ -35541,7 +35541,7 @@
       </c>
       <c r="B567" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C567" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -71749,7 +71749,7 @@
       </c>
       <c r="B1151" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1151" s="2" t="inlineStr">
@@ -73609,7 +73609,7 @@
       </c>
       <c r="B1181" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1181" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -74973,7 +74973,7 @@
       </c>
       <c r="B1203" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1203" s="2" t="inlineStr">
@@ -77577,7 +77577,7 @@
       </c>
       <c r="B1245" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1245" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84769,7 +84769,7 @@
       </c>
       <c r="B1361" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1361" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -86629,7 +86629,7 @@
       </c>
       <c r="B1391" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1391" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91031,7 +91031,7 @@
       </c>
       <c r="B1462" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1462" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -92643,7 +92643,7 @@
       </c>
       <c r="B1488" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 23:10:16
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -33185,7 +33185,7 @@
       </c>
       <c r="B529" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C529" s="2" t="inlineStr">
@@ -34921,7 +34921,7 @@
       </c>
       <c r="B557" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C557" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -42981,7 +42981,7 @@
       </c>
       <c r="B687" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C687" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -51599,7 +51599,7 @@
       </c>
       <c r="B826" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C826" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -58233,7 +58233,7 @@
       </c>
       <c r="B933" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C933" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71749,7 +71749,7 @@
       </c>
       <c r="B1151" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1151" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -74973,7 +74973,7 @@
       </c>
       <c r="B1203" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1203" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -79561,7 +79561,7 @@
       </c>
       <c r="B1277" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1277" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84769,7 +84769,7 @@
       </c>
       <c r="B1361" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1361" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -88489,7 +88489,7 @@
       </c>
       <c r="B1421" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1421" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91031,7 +91031,7 @@
       </c>
       <c r="B1462" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1462" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 23:20:34
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
@@ -33185,7 +33185,7 @@
       </c>
       <c r="B529" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C529" s="2" t="inlineStr">
@@ -34921,7 +34921,7 @@
       </c>
       <c r="B557" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C557" s="2" t="inlineStr">
@@ -35541,7 +35541,7 @@
       </c>
       <c r="B567" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C567" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="B612" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C612" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51599,7 +51599,7 @@
       </c>
       <c r="B826" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C826" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -74973,7 +74973,7 @@
       </c>
       <c r="B1203" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1203" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -79747,7 +79747,7 @@
       </c>
       <c r="B1280" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1280" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -84087,7 +84087,7 @@
       </c>
       <c r="B1350" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1350" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84769,7 +84769,7 @@
       </c>
       <c r="B1361" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1361" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 23:31:53
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
@@ -33185,7 +33185,7 @@
       </c>
       <c r="B529" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C529" s="2" t="inlineStr">
@@ -34921,7 +34921,7 @@
       </c>
       <c r="B557" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C557" s="2" t="inlineStr">
@@ -35541,7 +35541,7 @@
       </c>
       <c r="B567" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C567" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -74601,7 +74601,7 @@
       </c>
       <c r="B1197" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1197" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -77577,7 +77577,7 @@
       </c>
       <c r="B1245" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1245" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -79561,7 +79561,7 @@
       </c>
       <c r="B1277" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1277" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -84087,7 +84087,7 @@
       </c>
       <c r="B1350" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1350" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84769,7 +84769,7 @@
       </c>
       <c r="B1361" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1361" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 23:41:53
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -31573,7 +31573,7 @@
       </c>
       <c r="B503" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C503" s="2" t="inlineStr">
@@ -31635,7 +31635,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
@@ -34425,7 +34425,7 @@
       </c>
       <c r="B549" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C549" s="2" t="inlineStr">
@@ -34921,7 +34921,7 @@
       </c>
       <c r="B557" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C557" s="2" t="inlineStr">
@@ -35541,7 +35541,7 @@
       </c>
       <c r="B567" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C567" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="B612" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C612" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -51103,7 +51103,7 @@
       </c>
       <c r="B818" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C818" s="2" t="inlineStr">
@@ -51599,7 +51599,7 @@
       </c>
       <c r="B826" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C826" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -74601,7 +74601,7 @@
       </c>
       <c r="B1197" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1197" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -79375,7 +79375,7 @@
       </c>
       <c r="B1274" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1274" s="2" t="inlineStr">
@@ -79561,7 +79561,7 @@
       </c>
       <c r="B1277" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1277" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -92643,7 +92643,7 @@
       </c>
       <c r="B1488" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-12 23:51:08
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -30767,7 +30767,7 @@
       </c>
       <c r="B490" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C490" s="2" t="inlineStr">
@@ -31573,7 +31573,7 @@
       </c>
       <c r="B503" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C503" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
@@ -33185,7 +33185,7 @@
       </c>
       <c r="B529" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C529" s="2" t="inlineStr">
@@ -34921,7 +34921,7 @@
       </c>
       <c r="B557" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C557" s="2" t="inlineStr">
@@ -35541,7 +35541,7 @@
       </c>
       <c r="B567" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C567" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51103,7 +51103,7 @@
       </c>
       <c r="B818" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C818" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51599,7 +51599,7 @@
       </c>
       <c r="B826" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C826" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -58171,7 +58171,7 @@
       </c>
       <c r="B932" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C932" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -69641,7 +69641,7 @@
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -71749,7 +71749,7 @@
       </c>
       <c r="B1151" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1151" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -79375,7 +79375,7 @@
       </c>
       <c r="B1274" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1274" s="2" t="inlineStr">
@@ -83467,7 +83467,7 @@
       </c>
       <c r="B1340" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1340" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -86629,7 +86629,7 @@
       </c>
       <c r="B1391" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1391" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -87993,7 +87993,7 @@
       </c>
       <c r="B1413" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1413" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -91961,7 +91961,7 @@
       </c>
       <c r="B1477" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1477" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-13 00:01:46
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -33185,7 +33185,7 @@
       </c>
       <c r="B529" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C529" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -42981,7 +42981,7 @@
       </c>
       <c r="B687" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C687" s="2" t="inlineStr">
@@ -48933,7 +48933,7 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C783" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51103,7 +51103,7 @@
       </c>
       <c r="B818" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C818" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C825" s="2" t="inlineStr">
@@ -51599,7 +51599,7 @@
       </c>
       <c r="B826" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C826" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -63193,7 +63193,7 @@
       </c>
       <c r="B1013" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1013" s="2" t="inlineStr">
@@ -66789,7 +66789,7 @@
       </c>
       <c r="B1071" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1071" s="2" t="inlineStr">
@@ -69703,7 +69703,7 @@
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
@@ -71191,7 +71191,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71749,7 +71749,7 @@
       </c>
       <c r="B1151" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1151" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -74973,7 +74973,7 @@
       </c>
       <c r="B1203" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1203" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77577,7 +77577,7 @@
       </c>
       <c r="B1245" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1245" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -79375,7 +79375,7 @@
       </c>
       <c r="B1274" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1274" s="2" t="inlineStr">
@@ -79747,7 +79747,7 @@
       </c>
       <c r="B1280" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1280" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -86629,7 +86629,7 @@
       </c>
       <c r="B1391" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1391" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -88489,7 +88489,7 @@
       </c>
       <c r="B1421" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1421" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -92643,7 +92643,7 @@
       </c>
       <c r="B1488" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-13 00:10:38
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -34425,7 +34425,7 @@
       </c>
       <c r="B549" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C549" s="2" t="inlineStr">
@@ -35665,7 +35665,7 @@
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="B612" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C612" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="B681" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C681" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -42919,7 +42919,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -42981,7 +42981,7 @@
       </c>
       <c r="B687" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C687" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B710" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C710" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -51103,7 +51103,7 @@
       </c>
       <c r="B818" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C818" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -71563,7 +71563,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -74663,7 +74663,7 @@
       </c>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1198" s="2" t="inlineStr">
@@ -74725,7 +74725,7 @@
       </c>
       <c r="B1199" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1199" s="2" t="inlineStr">
@@ -74787,7 +74787,7 @@
       </c>
       <c r="B1200" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1200" s="2" t="inlineStr">
@@ -74973,7 +74973,7 @@
       </c>
       <c r="B1203" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1203" s="2" t="inlineStr">
@@ -75035,7 +75035,7 @@
       </c>
       <c r="B1204" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1204" s="2" t="inlineStr">
@@ -76213,7 +76213,7 @@
       </c>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1223" s="2" t="inlineStr">
@@ -77577,7 +77577,7 @@
       </c>
       <c r="B1245" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1245" s="2" t="inlineStr">
@@ -77639,7 +77639,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1246" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -78879,7 +78879,7 @@
       </c>
       <c r="B1266" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1266" s="2" t="inlineStr">
@@ -79375,7 +79375,7 @@
       </c>
       <c r="B1274" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1274" s="2" t="inlineStr">
@@ -83591,7 +83591,7 @@
       </c>
       <c r="B1342" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1342" s="2" t="inlineStr">
@@ -83653,7 +83653,7 @@
       </c>
       <c r="B1343" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1343" s="2" t="inlineStr">
@@ -83963,7 +83963,7 @@
       </c>
       <c r="B1348" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1348" s="2" t="inlineStr">
@@ -84087,7 +84087,7 @@
       </c>
       <c r="B1350" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1350" s="2" t="inlineStr">
@@ -84273,7 +84273,7 @@
       </c>
       <c r="B1353" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1353" s="2" t="inlineStr">
@@ -84707,7 +84707,7 @@
       </c>
       <c r="B1360" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1360" s="2" t="inlineStr">
@@ -84893,7 +84893,7 @@
       </c>
       <c r="B1363" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1363" s="2" t="inlineStr">
@@ -87931,7 +87931,7 @@
       </c>
       <c r="B1412" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1412" s="2" t="inlineStr">
@@ -88489,7 +88489,7 @@
       </c>
       <c r="B1421" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1421" s="2" t="inlineStr">
@@ -88551,7 +88551,7 @@
       </c>
       <c r="B1422" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1422" s="2" t="inlineStr">
@@ -90225,7 +90225,7 @@
       </c>
       <c r="B1449" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1449" s="2" t="inlineStr">
@@ -90287,7 +90287,7 @@
       </c>
       <c r="B1450" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1450" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -91961,7 +91961,7 @@
       </c>
       <c r="B1477" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1477" s="2" t="inlineStr">
@@ -92643,7 +92643,7 @@
       </c>
       <c r="B1488" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-13 00:30:43
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -31821,7 +31821,7 @@
       </c>
       <c r="B507" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C507" s="2" t="inlineStr">
@@ -37897,7 +37897,7 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="B612" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C612" s="2" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -42485,7 +42485,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -42733,7 +42733,7 @@
       </c>
       <c r="B683" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C683" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -43787,7 +43787,7 @@
       </c>
       <c r="B700" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C700" s="2" t="inlineStr">
@@ -47445,7 +47445,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -51041,7 +51041,7 @@
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C817" s="2" t="inlineStr">
@@ -51661,7 +51661,7 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C827" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -56001,7 +56001,7 @@
       </c>
       <c r="B897" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C897" s="2" t="inlineStr">
@@ -58233,7 +58233,7 @@
       </c>
       <c r="B933" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C933" s="2" t="inlineStr">
@@ -69579,7 +69579,7 @@
       </c>
       <c r="B1116" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1116" s="2" t="inlineStr">
@@ -69765,7 +69765,7 @@
       </c>
       <c r="B1119" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1119" s="2" t="inlineStr">
@@ -70137,7 +70137,7 @@
       </c>
       <c r="B1125" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1125" s="2" t="inlineStr">
@@ -70385,7 +70385,7 @@
       </c>
       <c r="B1129" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1129" s="2" t="inlineStr">
@@ -71315,7 +71315,7 @@
       </c>
       <c r="B1144" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1144" s="2" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
@@ -73733,7 +73733,7 @@
       </c>
       <c r="B1183" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1183" s="2" t="inlineStr">
@@ -74911,7 +74911,7 @@
       </c>
       <c r="B1202" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1202" s="2" t="inlineStr">
@@ -76337,7 +76337,7 @@
       </c>
       <c r="B1225" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1225" s="2" t="inlineStr">
@@ -77701,7 +77701,7 @@
       </c>
       <c r="B1247" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1247" s="2" t="inlineStr">
@@ -77763,7 +77763,7 @@
       </c>
       <c r="B1248" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1248" s="2" t="inlineStr">
@@ -79003,7 +79003,7 @@
       </c>
       <c r="B1268" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1268" s="2" t="inlineStr">
@@ -79685,7 +79685,7 @@
       </c>
       <c r="B1279" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1279" s="2" t="inlineStr">
@@ -79871,7 +79871,7 @@
       </c>
       <c r="B1282" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1282" s="2" t="inlineStr">
@@ -83715,7 +83715,7 @@
       </c>
       <c r="B1344" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1344" s="2" t="inlineStr">
@@ -84087,7 +84087,7 @@
       </c>
       <c r="B1350" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1350" s="2" t="inlineStr">
@@ -84397,7 +84397,7 @@
       </c>
       <c r="B1355" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1355" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84955,7 +84955,7 @@
       </c>
       <c r="B1364" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1364" s="2" t="inlineStr">
@@ -86753,7 +86753,7 @@
       </c>
       <c r="B1393" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1393" s="2" t="inlineStr">
@@ -88613,7 +88613,7 @@
       </c>
       <c r="B1423" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1423" s="2" t="inlineStr">
@@ -88675,7 +88675,7 @@
       </c>
       <c r="B1424" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1424" s="2" t="inlineStr">
@@ -90349,7 +90349,7 @@
       </c>
       <c r="B1451" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1451" s="2" t="inlineStr">
@@ -92767,7 +92767,7 @@
       </c>
       <c r="B1490" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1490" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-13 01:00:49
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7579,7 +7579,7 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
@@ -9191,7 +9191,7 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
@@ -15453,7 +15453,7 @@
       </c>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C243" s="2" t="inlineStr">
@@ -22707,7 +22707,7 @@
       </c>
       <c r="B360" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C360" s="2" t="inlineStr">
@@ -28659,7 +28659,7 @@
       </c>
       <c r="B456" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C456" s="2" t="inlineStr">
@@ -28721,7 +28721,7 @@
       </c>
       <c r="B457" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C457" s="2" t="inlineStr">
@@ -31945,7 +31945,7 @@
       </c>
       <c r="B509" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C509" s="2" t="inlineStr">
@@ -35851,7 +35851,7 @@
       </c>
       <c r="B572" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C572" s="2" t="inlineStr">
@@ -38207,7 +38207,7 @@
       </c>
       <c r="B610" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C610" s="2" t="inlineStr">
@@ -40625,7 +40625,7 @@
       </c>
       <c r="B649" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C649" s="2" t="inlineStr">
@@ -42919,7 +42919,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -43043,7 +43043,7 @@
       </c>
       <c r="B688" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C688" s="2" t="inlineStr">
@@ -43105,7 +43105,7 @@
       </c>
       <c r="B689" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C689" s="2" t="inlineStr">
@@ -44717,7 +44717,7 @@
       </c>
       <c r="B715" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C715" s="2" t="inlineStr">
@@ -47755,7 +47755,7 @@
       </c>
       <c r="B764" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C764" s="2" t="inlineStr">
@@ -51351,7 +51351,7 @@
       </c>
       <c r="B822" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C822" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -52033,7 +52033,7 @@
       </c>
       <c r="B833" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C833" s="2" t="inlineStr">
@@ -58543,7 +58543,7 @@
       </c>
       <c r="B938" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C938" s="2" t="inlineStr">
@@ -67223,7 +67223,7 @@
       </c>
       <c r="B1078" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1078" s="2" t="inlineStr">
@@ -71749,7 +71749,7 @@
       </c>
       <c r="B1151" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1151" s="2" t="inlineStr">
@@ -72121,7 +72121,7 @@
       </c>
       <c r="B1157" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1157" s="2" t="inlineStr">
@@ -72245,7 +72245,7 @@
       </c>
       <c r="B1159" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1159" s="2" t="inlineStr">
@@ -75221,7 +75221,7 @@
       </c>
       <c r="B1207" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1207" s="2" t="inlineStr">
@@ -76771,7 +76771,7 @@
       </c>
       <c r="B1232" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1232" s="2" t="inlineStr">
@@ -78135,7 +78135,7 @@
       </c>
       <c r="B1254" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1254" s="2" t="inlineStr">
@@ -78259,7 +78259,7 @@
       </c>
       <c r="B1256" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1256" s="2" t="inlineStr">
@@ -79127,7 +79127,7 @@
       </c>
       <c r="B1270" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1270" s="2" t="inlineStr">
@@ -79623,7 +79623,7 @@
       </c>
       <c r="B1278" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1278" s="2" t="inlineStr">
@@ -80119,7 +80119,7 @@
       </c>
       <c r="B1286" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1286" s="2" t="inlineStr">
@@ -80367,7 +80367,7 @@
       </c>
       <c r="B1290" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1290" s="2" t="inlineStr">
@@ -84335,7 +84335,7 @@
       </c>
       <c r="B1354" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1354" s="2" t="inlineStr">
@@ -84459,7 +84459,7 @@
       </c>
       <c r="B1356" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1356" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84583,7 +84583,7 @@
       </c>
       <c r="B1358" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1358" s="2" t="inlineStr">
@@ -85389,7 +85389,7 @@
       </c>
       <c r="B1371" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1371" s="2" t="inlineStr">
@@ -85637,7 +85637,7 @@
       </c>
       <c r="B1375" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1375" s="2" t="inlineStr">
@@ -88799,7 +88799,7 @@
       </c>
       <c r="B1426" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1426" s="2" t="inlineStr">
@@ -89543,7 +89543,7 @@
       </c>
       <c r="B1438" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1438" s="2" t="inlineStr">
@@ -91217,7 +91217,7 @@
       </c>
       <c r="B1465" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1465" s="2" t="inlineStr">
@@ -92953,7 +92953,7 @@
       </c>
       <c r="B1493" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1493" s="2" t="inlineStr">
@@ -93635,7 +93635,7 @@
       </c>
       <c r="B1504" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1504" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-13 01:10:33
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -8075,7 +8075,7 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
@@ -22707,7 +22707,7 @@
       </c>
       <c r="B360" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C360" s="2" t="inlineStr">
@@ -28659,7 +28659,7 @@
       </c>
       <c r="B456" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C456" s="2" t="inlineStr">
@@ -28721,7 +28721,7 @@
       </c>
       <c r="B457" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C457" s="2" t="inlineStr">
@@ -31077,7 +31077,7 @@
       </c>
       <c r="B495" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C495" s="2" t="inlineStr">
@@ -34735,7 +34735,7 @@
       </c>
       <c r="B554" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C554" s="2" t="inlineStr">
@@ -42919,7 +42919,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -43105,7 +43105,7 @@
       </c>
       <c r="B689" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C689" s="2" t="inlineStr">
@@ -43291,7 +43291,7 @@
       </c>
       <c r="B692" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C692" s="2" t="inlineStr">
@@ -44717,7 +44717,7 @@
       </c>
       <c r="B715" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C715" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -51847,7 +51847,7 @@
       </c>
       <c r="B830" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C830" s="2" t="inlineStr">
@@ -51909,7 +51909,7 @@
       </c>
       <c r="B831" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C831" s="2" t="inlineStr">
@@ -51971,7 +51971,7 @@
       </c>
       <c r="B832" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C832" s="2" t="inlineStr">
@@ -58481,7 +58481,7 @@
       </c>
       <c r="B937" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C937" s="2" t="inlineStr">
@@ -58543,7 +58543,7 @@
       </c>
       <c r="B938" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C938" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -60651,7 +60651,7 @@
       </c>
       <c r="B972" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C972" s="2" t="inlineStr">
@@ -61023,7 +61023,7 @@
       </c>
       <c r="B978" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C978" s="2" t="inlineStr">
@@ -70199,7 +70199,7 @@
       </c>
       <c r="B1126" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1126" s="2" t="inlineStr">
@@ -70819,7 +70819,7 @@
       </c>
       <c r="B1136" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1136" s="2" t="inlineStr">
@@ -71749,7 +71749,7 @@
       </c>
       <c r="B1151" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1151" s="2" t="inlineStr">
@@ -72121,7 +72121,7 @@
       </c>
       <c r="B1157" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1157" s="2" t="inlineStr">
@@ -72245,7 +72245,7 @@
       </c>
       <c r="B1159" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1159" s="2" t="inlineStr">
@@ -72307,7 +72307,7 @@
       </c>
       <c r="B1160" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1160" s="2" t="inlineStr">
@@ -75221,7 +75221,7 @@
       </c>
       <c r="B1207" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1207" s="2" t="inlineStr">
@@ -75593,7 +75593,7 @@
       </c>
       <c r="B1213" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1213" s="2" t="inlineStr">
@@ -79127,7 +79127,7 @@
       </c>
       <c r="B1270" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1270" s="2" t="inlineStr">
@@ -79623,7 +79623,7 @@
       </c>
       <c r="B1278" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1278" s="2" t="inlineStr">
@@ -80119,7 +80119,7 @@
       </c>
       <c r="B1286" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1286" s="2" t="inlineStr">
@@ -80367,7 +80367,7 @@
       </c>
       <c r="B1290" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1290" s="2" t="inlineStr">
@@ -80429,7 +80429,7 @@
       </c>
       <c r="B1291" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1291" s="2" t="inlineStr">
@@ -84335,7 +84335,7 @@
       </c>
       <c r="B1354" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1354" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84583,7 +84583,7 @@
       </c>
       <c r="B1358" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1358" s="2" t="inlineStr">
@@ -84955,7 +84955,7 @@
       </c>
       <c r="B1364" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1364" s="2" t="inlineStr">
@@ -85141,7 +85141,7 @@
       </c>
       <c r="B1367" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1367" s="2" t="inlineStr">
@@ -85389,7 +85389,7 @@
       </c>
       <c r="B1371" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1371" s="2" t="inlineStr">
@@ -85637,7 +85637,7 @@
       </c>
       <c r="B1375" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1375" s="2" t="inlineStr">
@@ -85699,7 +85699,7 @@
       </c>
       <c r="B1376" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1376" s="2" t="inlineStr">
@@ -87497,7 +87497,7 @@
       </c>
       <c r="B1405" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1405" s="2" t="inlineStr">
@@ -88799,7 +88799,7 @@
       </c>
       <c r="B1426" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1426" s="2" t="inlineStr">
@@ -88861,7 +88861,7 @@
       </c>
       <c r="B1427" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1427" s="2" t="inlineStr">
@@ -89171,7 +89171,7 @@
       </c>
       <c r="B1432" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1432" s="2" t="inlineStr">
@@ -89543,7 +89543,7 @@
       </c>
       <c r="B1438" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1438" s="2" t="inlineStr">
@@ -91217,7 +91217,7 @@
       </c>
       <c r="B1465" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1465" s="2" t="inlineStr">
@@ -91341,7 +91341,7 @@
       </c>
       <c r="B1467" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1467" s="2" t="inlineStr">
@@ -92271,7 +92271,7 @@
       </c>
       <c r="B1482" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1482" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-13 01:20:47
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -7579,7 +7579,7 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
@@ -8075,7 +8075,7 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
@@ -9191,7 +9191,7 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
@@ -15453,7 +15453,7 @@
       </c>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C243" s="2" t="inlineStr">
@@ -28659,7 +28659,7 @@
       </c>
       <c r="B456" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C456" s="2" t="inlineStr">
@@ -28721,7 +28721,7 @@
       </c>
       <c r="B457" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C457" s="2" t="inlineStr">
@@ -29341,7 +29341,7 @@
       </c>
       <c r="B467" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C467" s="2" t="inlineStr">
@@ -33247,7 +33247,7 @@
       </c>
       <c r="B530" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C530" s="2" t="inlineStr">
@@ -34735,7 +34735,7 @@
       </c>
       <c r="B554" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C554" s="2" t="inlineStr">
@@ -35851,7 +35851,7 @@
       </c>
       <c r="B572" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C572" s="2" t="inlineStr">
@@ -35975,7 +35975,7 @@
       </c>
       <c r="B574" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C574" s="2" t="inlineStr">
@@ -38207,7 +38207,7 @@
       </c>
       <c r="B610" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C610" s="2" t="inlineStr">
@@ -38641,7 +38641,7 @@
       </c>
       <c r="B617" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C617" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -42919,7 +42919,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -43043,7 +43043,7 @@
       </c>
       <c r="B688" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C688" s="2" t="inlineStr">
@@ -44097,7 +44097,7 @@
       </c>
       <c r="B705" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C705" s="2" t="inlineStr">
@@ -44717,7 +44717,7 @@
       </c>
       <c r="B715" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C715" s="2" t="inlineStr">
@@ -47755,7 +47755,7 @@
       </c>
       <c r="B764" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C764" s="2" t="inlineStr">
@@ -49243,7 +49243,7 @@
       </c>
       <c r="B788" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C788" s="2" t="inlineStr">
@@ -51847,7 +51847,7 @@
       </c>
       <c r="B830" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C830" s="2" t="inlineStr">
@@ -52033,7 +52033,7 @@
       </c>
       <c r="B833" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C833" s="2" t="inlineStr">
@@ -58543,7 +58543,7 @@
       </c>
       <c r="B938" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C938" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -61023,7 +61023,7 @@
       </c>
       <c r="B978" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C978" s="2" t="inlineStr">
@@ -63627,7 +63627,7 @@
       </c>
       <c r="B1020" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1020" s="2" t="inlineStr">
@@ -67223,7 +67223,7 @@
       </c>
       <c r="B1078" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1078" s="2" t="inlineStr">
@@ -70199,7 +70199,7 @@
       </c>
       <c r="B1126" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1126" s="2" t="inlineStr">
@@ -70571,7 +70571,7 @@
       </c>
       <c r="B1132" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1132" s="2" t="inlineStr">
@@ -70819,7 +70819,7 @@
       </c>
       <c r="B1136" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1136" s="2" t="inlineStr">
@@ -71749,7 +71749,7 @@
       </c>
       <c r="B1151" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1151" s="2" t="inlineStr">
@@ -72121,7 +72121,7 @@
       </c>
       <c r="B1157" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1157" s="2" t="inlineStr">
@@ -72307,7 +72307,7 @@
       </c>
       <c r="B1160" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1160" s="2" t="inlineStr">
@@ -74167,7 +74167,7 @@
       </c>
       <c r="B1190" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1190" s="2" t="inlineStr">
@@ -75221,7 +75221,7 @@
       </c>
       <c r="B1207" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1207" s="2" t="inlineStr">
@@ -75283,7 +75283,7 @@
       </c>
       <c r="B1208" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1208" s="2" t="inlineStr">
@@ -78197,7 +78197,7 @@
       </c>
       <c r="B1255" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1255" s="2" t="inlineStr">
@@ -78259,7 +78259,7 @@
       </c>
       <c r="B1256" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1256" s="2" t="inlineStr">
@@ -79127,7 +79127,7 @@
       </c>
       <c r="B1270" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1270" s="2" t="inlineStr">
@@ -80119,7 +80119,7 @@
       </c>
       <c r="B1286" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1286" s="2" t="inlineStr">
@@ -80305,7 +80305,7 @@
       </c>
       <c r="B1289" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1289" s="2" t="inlineStr">
@@ -80429,7 +80429,7 @@
       </c>
       <c r="B1291" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1291" s="2" t="inlineStr">
@@ -84335,7 +84335,7 @@
       </c>
       <c r="B1354" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1354" s="2" t="inlineStr">
@@ -84459,7 +84459,7 @@
       </c>
       <c r="B1356" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1356" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -85141,7 +85141,7 @@
       </c>
       <c r="B1367" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1367" s="2" t="inlineStr">
@@ -85265,7 +85265,7 @@
       </c>
       <c r="B1369" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1369" s="2" t="inlineStr">
@@ -85637,7 +85637,7 @@
       </c>
       <c r="B1375" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1375" s="2" t="inlineStr">
@@ -87497,7 +87497,7 @@
       </c>
       <c r="B1405" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1405" s="2" t="inlineStr">
@@ -88861,7 +88861,7 @@
       </c>
       <c r="B1427" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1427" s="2" t="inlineStr">
@@ -89171,7 +89171,7 @@
       </c>
       <c r="B1432" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1432" s="2" t="inlineStr">
@@ -91341,7 +91341,7 @@
       </c>
       <c r="B1467" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1467" s="2" t="inlineStr">
@@ -92023,7 +92023,7 @@
       </c>
       <c r="B1478" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1478" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-13 01:30:30
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7579,7 +7579,7 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
@@ -8075,7 +8075,7 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
@@ -9191,7 +9191,7 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
@@ -15453,7 +15453,7 @@
       </c>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C243" s="2" t="inlineStr">
@@ -22459,7 +22459,7 @@
       </c>
       <c r="B356" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C356" s="2" t="inlineStr">
@@ -28659,7 +28659,7 @@
       </c>
       <c r="B456" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C456" s="2" t="inlineStr">
@@ -31077,7 +31077,7 @@
       </c>
       <c r="B495" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C495" s="2" t="inlineStr">
@@ -31945,7 +31945,7 @@
       </c>
       <c r="B509" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C509" s="2" t="inlineStr">
@@ -32131,7 +32131,7 @@
       </c>
       <c r="B512" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C512" s="2" t="inlineStr">
@@ -33247,7 +33247,7 @@
       </c>
       <c r="B530" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C530" s="2" t="inlineStr">
@@ -34735,7 +34735,7 @@
       </c>
       <c r="B554" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C554" s="2" t="inlineStr">
@@ -35851,7 +35851,7 @@
       </c>
       <c r="B572" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C572" s="2" t="inlineStr">
@@ -42919,7 +42919,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -43043,7 +43043,7 @@
       </c>
       <c r="B688" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C688" s="2" t="inlineStr">
@@ -43105,7 +43105,7 @@
       </c>
       <c r="B689" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C689" s="2" t="inlineStr">
@@ -44717,7 +44717,7 @@
       </c>
       <c r="B715" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C715" s="2" t="inlineStr">
@@ -47755,7 +47755,7 @@
       </c>
       <c r="B764" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C764" s="2" t="inlineStr">
@@ -49243,7 +49243,7 @@
       </c>
       <c r="B788" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C788" s="2" t="inlineStr">
@@ -51351,7 +51351,7 @@
       </c>
       <c r="B822" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C822" s="2" t="inlineStr">
@@ -51847,7 +51847,7 @@
       </c>
       <c r="B830" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C830" s="2" t="inlineStr">
@@ -51971,7 +51971,7 @@
       </c>
       <c r="B832" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C832" s="2" t="inlineStr">
@@ -52033,7 +52033,7 @@
       </c>
       <c r="B833" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C833" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -60651,7 +60651,7 @@
       </c>
       <c r="B972" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C972" s="2" t="inlineStr">
@@ -61023,7 +61023,7 @@
       </c>
       <c r="B978" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C978" s="2" t="inlineStr">
@@ -63627,7 +63627,7 @@
       </c>
       <c r="B1020" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1020" s="2" t="inlineStr">
@@ -70571,7 +70571,7 @@
       </c>
       <c r="B1132" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1132" s="2" t="inlineStr">
@@ -70819,7 +70819,7 @@
       </c>
       <c r="B1136" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1136" s="2" t="inlineStr">
@@ -71749,7 +71749,7 @@
       </c>
       <c r="B1151" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1151" s="2" t="inlineStr">
@@ -72121,7 +72121,7 @@
       </c>
       <c r="B1157" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1157" s="2" t="inlineStr">
@@ -72245,7 +72245,7 @@
       </c>
       <c r="B1159" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1159" s="2" t="inlineStr">
@@ -75283,7 +75283,7 @@
       </c>
       <c r="B1208" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1208" s="2" t="inlineStr">
@@ -75345,7 +75345,7 @@
       </c>
       <c r="B1209" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1209" s="2" t="inlineStr">
@@ -75593,7 +75593,7 @@
       </c>
       <c r="B1213" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1213" s="2" t="inlineStr">
@@ -78259,7 +78259,7 @@
       </c>
       <c r="B1256" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1256" s="2" t="inlineStr">
@@ -79127,7 +79127,7 @@
       </c>
       <c r="B1270" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1270" s="2" t="inlineStr">
@@ -80119,7 +80119,7 @@
       </c>
       <c r="B1286" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1286" s="2" t="inlineStr">
@@ -84459,7 +84459,7 @@
       </c>
       <c r="B1356" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1356" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -84955,7 +84955,7 @@
       </c>
       <c r="B1364" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1364" s="2" t="inlineStr">
@@ -85141,7 +85141,7 @@
       </c>
       <c r="B1367" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1367" s="2" t="inlineStr">
@@ -85575,7 +85575,7 @@
       </c>
       <c r="B1374" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1374" s="2" t="inlineStr">
@@ -85637,7 +85637,7 @@
       </c>
       <c r="B1375" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1375" s="2" t="inlineStr">
@@ -87497,7 +87497,7 @@
       </c>
       <c r="B1405" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1405" s="2" t="inlineStr">
@@ -88861,7 +88861,7 @@
       </c>
       <c r="B1427" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1427" s="2" t="inlineStr">
@@ -89171,7 +89171,7 @@
       </c>
       <c r="B1432" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1432" s="2" t="inlineStr">
@@ -89543,7 +89543,7 @@
       </c>
       <c r="B1438" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1438" s="2" t="inlineStr">
@@ -92023,7 +92023,7 @@
       </c>
       <c r="B1478" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1478" s="2" t="inlineStr">
@@ -92953,7 +92953,7 @@
       </c>
       <c r="B1493" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1493" s="2" t="inlineStr">
@@ -93635,7 +93635,7 @@
       </c>
       <c r="B1504" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1504" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-13 01:41:09
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -7455,7 +7455,7 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -7517,7 +7517,7 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
@@ -7579,7 +7579,7 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
@@ -8075,7 +8075,7 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
@@ -8757,7 +8757,7 @@
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
@@ -9191,7 +9191,7 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
@@ -15453,7 +15453,7 @@
       </c>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C243" s="2" t="inlineStr">
@@ -28659,7 +28659,7 @@
       </c>
       <c r="B456" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C456" s="2" t="inlineStr">
@@ -30023,7 +30023,7 @@
       </c>
       <c r="B478" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C478" s="2" t="inlineStr">
@@ -31945,7 +31945,7 @@
       </c>
       <c r="B509" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C509" s="2" t="inlineStr">
@@ -32131,7 +32131,7 @@
       </c>
       <c r="B512" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C512" s="2" t="inlineStr">
@@ -34735,7 +34735,7 @@
       </c>
       <c r="B554" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C554" s="2" t="inlineStr">
@@ -38641,7 +38641,7 @@
       </c>
       <c r="B617" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C617" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -43043,7 +43043,7 @@
       </c>
       <c r="B688" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C688" s="2" t="inlineStr">
@@ -43291,7 +43291,7 @@
       </c>
       <c r="B692" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C692" s="2" t="inlineStr">
@@ -44717,7 +44717,7 @@
       </c>
       <c r="B715" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C715" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -51847,7 +51847,7 @@
       </c>
       <c r="B830" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C830" s="2" t="inlineStr">
@@ -51909,7 +51909,7 @@
       </c>
       <c r="B831" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C831" s="2" t="inlineStr">
@@ -51971,7 +51971,7 @@
       </c>
       <c r="B832" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C832" s="2" t="inlineStr">
@@ -52033,7 +52033,7 @@
       </c>
       <c r="B833" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C833" s="2" t="inlineStr">
@@ -60651,7 +60651,7 @@
       </c>
       <c r="B972" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C972" s="2" t="inlineStr">
@@ -61023,7 +61023,7 @@
       </c>
       <c r="B978" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C978" s="2" t="inlineStr">
@@ -63627,7 +63627,7 @@
       </c>
       <c r="B1020" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1020" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -70199,7 +70199,7 @@
       </c>
       <c r="B1126" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1126" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -70819,7 +70819,7 @@
       </c>
       <c r="B1136" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1136" s="2" t="inlineStr">
@@ -72121,7 +72121,7 @@
       </c>
       <c r="B1157" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1157" s="2" t="inlineStr">
@@ -72245,7 +72245,7 @@
       </c>
       <c r="B1159" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1159" s="2" t="inlineStr">
@@ -74167,7 +74167,7 @@
       </c>
       <c r="B1190" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1190" s="2" t="inlineStr">
@@ -75221,7 +75221,7 @@
       </c>
       <c r="B1207" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1207" s="2" t="inlineStr">
@@ -75345,7 +75345,7 @@
       </c>
       <c r="B1209" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1209" s="2" t="inlineStr">
@@ -75593,7 +75593,7 @@
       </c>
       <c r="B1213" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1213" s="2" t="inlineStr">
@@ -79127,7 +79127,7 @@
       </c>
       <c r="B1270" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1270" s="2" t="inlineStr">
@@ -79189,7 +79189,7 @@
       </c>
       <c r="B1271" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1271" s="2" t="inlineStr">
@@ -79623,7 +79623,7 @@
       </c>
       <c r="B1278" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1278" s="2" t="inlineStr">
@@ -80429,7 +80429,7 @@
       </c>
       <c r="B1291" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1291" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -84955,7 +84955,7 @@
       </c>
       <c r="B1364" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1364" s="2" t="inlineStr">
@@ -85265,7 +85265,7 @@
       </c>
       <c r="B1369" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1369" s="2" t="inlineStr">
@@ -85389,7 +85389,7 @@
       </c>
       <c r="B1371" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1371" s="2" t="inlineStr">
@@ -85575,7 +85575,7 @@
       </c>
       <c r="B1374" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1374" s="2" t="inlineStr">
@@ -85699,7 +85699,7 @@
       </c>
       <c r="B1376" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1376" s="2" t="inlineStr">
@@ -87497,7 +87497,7 @@
       </c>
       <c r="B1405" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1405" s="2" t="inlineStr">
@@ -88861,7 +88861,7 @@
       </c>
       <c r="B1427" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1427" s="2" t="inlineStr">
@@ -89543,7 +89543,7 @@
       </c>
       <c r="B1438" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1438" s="2" t="inlineStr">
@@ -91217,7 +91217,7 @@
       </c>
       <c r="B1465" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1465" s="2" t="inlineStr">
@@ -92271,7 +92271,7 @@
       </c>
       <c r="B1482" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1482" s="2" t="inlineStr">
@@ -93635,7 +93635,7 @@
       </c>
       <c r="B1504" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1504" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-13 01:51:10
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7455,7 +7455,7 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -7517,7 +7517,7 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
@@ -7579,7 +7579,7 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
@@ -15453,7 +15453,7 @@
       </c>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C243" s="2" t="inlineStr">
@@ -22459,7 +22459,7 @@
       </c>
       <c r="B356" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C356" s="2" t="inlineStr">
@@ -28659,7 +28659,7 @@
       </c>
       <c r="B456" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C456" s="2" t="inlineStr">
@@ -28721,7 +28721,7 @@
       </c>
       <c r="B457" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C457" s="2" t="inlineStr">
@@ -29341,7 +29341,7 @@
       </c>
       <c r="B467" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C467" s="2" t="inlineStr">
@@ -30023,7 +30023,7 @@
       </c>
       <c r="B478" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C478" s="2" t="inlineStr">
@@ -31077,7 +31077,7 @@
       </c>
       <c r="B495" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C495" s="2" t="inlineStr">
@@ -32131,7 +32131,7 @@
       </c>
       <c r="B512" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C512" s="2" t="inlineStr">
@@ -35851,7 +35851,7 @@
       </c>
       <c r="B572" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C572" s="2" t="inlineStr">
@@ -35975,7 +35975,7 @@
       </c>
       <c r="B574" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C574" s="2" t="inlineStr">
@@ -40625,7 +40625,7 @@
       </c>
       <c r="B649" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C649" s="2" t="inlineStr">
@@ -42919,7 +42919,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -43043,7 +43043,7 @@
       </c>
       <c r="B688" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C688" s="2" t="inlineStr">
@@ -43105,7 +43105,7 @@
       </c>
       <c r="B689" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C689" s="2" t="inlineStr">
@@ -43291,7 +43291,7 @@
       </c>
       <c r="B692" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C692" s="2" t="inlineStr">
@@ -44097,7 +44097,7 @@
       </c>
       <c r="B705" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C705" s="2" t="inlineStr">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -51847,7 +51847,7 @@
       </c>
       <c r="B830" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C830" s="2" t="inlineStr">
@@ -51971,7 +51971,7 @@
       </c>
       <c r="B832" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C832" s="2" t="inlineStr">
@@ -52033,7 +52033,7 @@
       </c>
       <c r="B833" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C833" s="2" t="inlineStr">
@@ -56311,7 +56311,7 @@
       </c>
       <c r="B902" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C902" s="2" t="inlineStr">
@@ -58481,7 +58481,7 @@
       </c>
       <c r="B937" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C937" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -60651,7 +60651,7 @@
       </c>
       <c r="B972" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C972" s="2" t="inlineStr">
@@ -61023,7 +61023,7 @@
       </c>
       <c r="B978" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C978" s="2" t="inlineStr">
@@ -70199,7 +70199,7 @@
       </c>
       <c r="B1126" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1126" s="2" t="inlineStr">
@@ -70571,7 +70571,7 @@
       </c>
       <c r="B1132" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1132" s="2" t="inlineStr">
@@ -72121,7 +72121,7 @@
       </c>
       <c r="B1157" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1157" s="2" t="inlineStr">
@@ -74167,7 +74167,7 @@
       </c>
       <c r="B1190" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1190" s="2" t="inlineStr">
@@ -75221,7 +75221,7 @@
       </c>
       <c r="B1207" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1207" s="2" t="inlineStr">
@@ -75345,7 +75345,7 @@
       </c>
       <c r="B1209" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1209" s="2" t="inlineStr">
@@ -78197,7 +78197,7 @@
       </c>
       <c r="B1255" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1255" s="2" t="inlineStr">
@@ -78321,7 +78321,7 @@
       </c>
       <c r="B1257" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1257" s="2" t="inlineStr">
@@ -79189,7 +79189,7 @@
       </c>
       <c r="B1271" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1271" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84583,7 +84583,7 @@
       </c>
       <c r="B1358" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1358" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -84955,7 +84955,7 @@
       </c>
       <c r="B1364" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1364" s="2" t="inlineStr">
@@ -85141,7 +85141,7 @@
       </c>
       <c r="B1367" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1367" s="2" t="inlineStr">
@@ -85575,7 +85575,7 @@
       </c>
       <c r="B1374" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1374" s="2" t="inlineStr">
@@ -85637,7 +85637,7 @@
       </c>
       <c r="B1375" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1375" s="2" t="inlineStr">
@@ -85699,7 +85699,7 @@
       </c>
       <c r="B1376" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1376" s="2" t="inlineStr">
@@ -85761,7 +85761,7 @@
       </c>
       <c r="B1377" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1377" s="2" t="inlineStr">
@@ -89543,7 +89543,7 @@
       </c>
       <c r="B1438" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1438" s="2" t="inlineStr">
@@ -91217,7 +91217,7 @@
       </c>
       <c r="B1465" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1465" s="2" t="inlineStr">
@@ -92023,7 +92023,7 @@
       </c>
       <c r="B1478" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1478" s="2" t="inlineStr">
@@ -92271,7 +92271,7 @@
       </c>
       <c r="B1482" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1482" s="2" t="inlineStr">
@@ -93635,7 +93635,7 @@
       </c>
       <c r="B1504" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1504" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-13 02:01:19
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7517,7 +7517,7 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
@@ -7579,7 +7579,7 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
@@ -8757,7 +8757,7 @@
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
@@ -9191,7 +9191,7 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
@@ -28721,7 +28721,7 @@
       </c>
       <c r="B457" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C457" s="2" t="inlineStr">
@@ -30023,7 +30023,7 @@
       </c>
       <c r="B478" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C478" s="2" t="inlineStr">
@@ -31077,7 +31077,7 @@
       </c>
       <c r="B495" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C495" s="2" t="inlineStr">
@@ -31945,7 +31945,7 @@
       </c>
       <c r="B509" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C509" s="2" t="inlineStr">
@@ -32131,7 +32131,7 @@
       </c>
       <c r="B512" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C512" s="2" t="inlineStr">
@@ -33247,7 +33247,7 @@
       </c>
       <c r="B530" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C530" s="2" t="inlineStr">
@@ -35851,7 +35851,7 @@
       </c>
       <c r="B572" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C572" s="2" t="inlineStr">
@@ -38207,7 +38207,7 @@
       </c>
       <c r="B610" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C610" s="2" t="inlineStr">
@@ -38641,7 +38641,7 @@
       </c>
       <c r="B617" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C617" s="2" t="inlineStr">
@@ -40625,7 +40625,7 @@
       </c>
       <c r="B649" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C649" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -43043,7 +43043,7 @@
       </c>
       <c r="B688" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C688" s="2" t="inlineStr">
@@ -43291,7 +43291,7 @@
       </c>
       <c r="B692" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C692" s="2" t="inlineStr">
@@ -44717,7 +44717,7 @@
       </c>
       <c r="B715" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C715" s="2" t="inlineStr">
@@ -47755,7 +47755,7 @@
       </c>
       <c r="B764" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C764" s="2" t="inlineStr">
@@ -49243,7 +49243,7 @@
       </c>
       <c r="B788" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C788" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -51847,7 +51847,7 @@
       </c>
       <c r="B830" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C830" s="2" t="inlineStr">
@@ -51909,7 +51909,7 @@
       </c>
       <c r="B831" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C831" s="2" t="inlineStr">
@@ -51971,7 +51971,7 @@
       </c>
       <c r="B832" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C832" s="2" t="inlineStr">
@@ -52033,7 +52033,7 @@
       </c>
       <c r="B833" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C833" s="2" t="inlineStr">
@@ -56311,7 +56311,7 @@
       </c>
       <c r="B902" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C902" s="2" t="inlineStr">
@@ -58481,7 +58481,7 @@
       </c>
       <c r="B937" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C937" s="2" t="inlineStr">
@@ -58543,7 +58543,7 @@
       </c>
       <c r="B938" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C938" s="2" t="inlineStr">
@@ -61023,7 +61023,7 @@
       </c>
       <c r="B978" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C978" s="2" t="inlineStr">
@@ -63627,7 +63627,7 @@
       </c>
       <c r="B1020" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1020" s="2" t="inlineStr">
@@ -67223,7 +67223,7 @@
       </c>
       <c r="B1078" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1078" s="2" t="inlineStr">
@@ -70199,7 +70199,7 @@
       </c>
       <c r="B1126" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1126" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -72121,7 +72121,7 @@
       </c>
       <c r="B1157" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1157" s="2" t="inlineStr">
@@ -74167,7 +74167,7 @@
       </c>
       <c r="B1190" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1190" s="2" t="inlineStr">
@@ -75221,7 +75221,7 @@
       </c>
       <c r="B1207" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1207" s="2" t="inlineStr">
@@ -75531,7 +75531,7 @@
       </c>
       <c r="B1212" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1212" s="2" t="inlineStr">
@@ -75593,7 +75593,7 @@
       </c>
       <c r="B1213" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1213" s="2" t="inlineStr">
@@ -78259,7 +78259,7 @@
       </c>
       <c r="B1256" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1256" s="2" t="inlineStr">
@@ -78321,7 +78321,7 @@
       </c>
       <c r="B1257" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1257" s="2" t="inlineStr">
@@ -79189,7 +79189,7 @@
       </c>
       <c r="B1271" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1271" s="2" t="inlineStr">
@@ -80119,7 +80119,7 @@
       </c>
       <c r="B1286" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1286" s="2" t="inlineStr">
@@ -80305,7 +80305,7 @@
       </c>
       <c r="B1289" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1289" s="2" t="inlineStr">
@@ -80367,7 +80367,7 @@
       </c>
       <c r="B1290" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1290" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -85265,7 +85265,7 @@
       </c>
       <c r="B1369" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1369" s="2" t="inlineStr">
@@ -85637,7 +85637,7 @@
       </c>
       <c r="B1375" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1375" s="2" t="inlineStr">
@@ -85761,7 +85761,7 @@
       </c>
       <c r="B1377" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1377" s="2" t="inlineStr">
@@ -88799,7 +88799,7 @@
       </c>
       <c r="B1426" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1426" s="2" t="inlineStr">
@@ -88861,7 +88861,7 @@
       </c>
       <c r="B1427" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1427" s="2" t="inlineStr">
@@ -89171,7 +89171,7 @@
       </c>
       <c r="B1432" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1432" s="2" t="inlineStr">
@@ -89233,7 +89233,7 @@
       </c>
       <c r="B1433" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1433" s="2" t="inlineStr">
@@ -89481,7 +89481,7 @@
       </c>
       <c r="B1437" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1437" s="2" t="inlineStr">
@@ -91217,7 +91217,7 @@
       </c>
       <c r="B1465" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1465" s="2" t="inlineStr">
@@ -91341,7 +91341,7 @@
       </c>
       <c r="B1467" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1467" s="2" t="inlineStr">
@@ -92023,7 +92023,7 @@
       </c>
       <c r="B1478" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1478" s="2" t="inlineStr">
@@ -92271,7 +92271,7 @@
       </c>
       <c r="B1482" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1482" s="2" t="inlineStr">
@@ -92953,7 +92953,7 @@
       </c>
       <c r="B1493" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1493" s="2" t="inlineStr">
@@ -93635,7 +93635,7 @@
       </c>
       <c r="B1504" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1504" s="2" t="inlineStr">
@@ -93697,7 +93697,7 @@
       </c>
       <c r="B1505" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1505" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-13 02:11:38
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7517,7 +7517,7 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
@@ -7579,7 +7579,7 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
@@ -9191,7 +9191,7 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
@@ -22707,7 +22707,7 @@
       </c>
       <c r="B360" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C360" s="2" t="inlineStr">
@@ -28659,7 +28659,7 @@
       </c>
       <c r="B456" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C456" s="2" t="inlineStr">
@@ -28721,7 +28721,7 @@
       </c>
       <c r="B457" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C457" s="2" t="inlineStr">
@@ -29341,7 +29341,7 @@
       </c>
       <c r="B467" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C467" s="2" t="inlineStr">
@@ -30023,7 +30023,7 @@
       </c>
       <c r="B478" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C478" s="2" t="inlineStr">
@@ -31945,7 +31945,7 @@
       </c>
       <c r="B509" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C509" s="2" t="inlineStr">
@@ -33247,7 +33247,7 @@
       </c>
       <c r="B530" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C530" s="2" t="inlineStr">
@@ -35231,7 +35231,7 @@
       </c>
       <c r="B562" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C562" s="2" t="inlineStr">
@@ -38207,7 +38207,7 @@
       </c>
       <c r="B610" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C610" s="2" t="inlineStr">
@@ -40625,7 +40625,7 @@
       </c>
       <c r="B649" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C649" s="2" t="inlineStr">
@@ -42795,7 +42795,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C684" s="2" t="inlineStr">
@@ -43105,7 +43105,7 @@
       </c>
       <c r="B689" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C689" s="2" t="inlineStr">
@@ -44097,7 +44097,7 @@
       </c>
       <c r="B705" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C705" s="2" t="inlineStr">
@@ -44717,7 +44717,7 @@
       </c>
       <c r="B715" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C715" s="2" t="inlineStr">
@@ -47755,7 +47755,7 @@
       </c>
       <c r="B764" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C764" s="2" t="inlineStr">
@@ -49243,7 +49243,7 @@
       </c>
       <c r="B788" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C788" s="2" t="inlineStr">
@@ -51351,7 +51351,7 @@
       </c>
       <c r="B822" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C822" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -52033,7 +52033,7 @@
       </c>
       <c r="B833" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C833" s="2" t="inlineStr">
@@ -58481,7 +58481,7 @@
       </c>
       <c r="B937" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C937" s="2" t="inlineStr">
@@ -58543,7 +58543,7 @@
       </c>
       <c r="B938" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C938" s="2" t="inlineStr">
@@ -60589,7 +60589,7 @@
       </c>
       <c r="B971" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C971" s="2" t="inlineStr">
@@ -70013,7 +70013,7 @@
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
@@ -70199,7 +70199,7 @@
       </c>
       <c r="B1126" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1126" s="2" t="inlineStr">
@@ -71749,7 +71749,7 @@
       </c>
       <c r="B1151" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1151" s="2" t="inlineStr">
@@ -72245,7 +72245,7 @@
       </c>
       <c r="B1159" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1159" s="2" t="inlineStr">
@@ -75221,7 +75221,7 @@
       </c>
       <c r="B1207" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1207" s="2" t="inlineStr">
@@ -75345,7 +75345,7 @@
       </c>
       <c r="B1209" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1209" s="2" t="inlineStr">
@@ -75531,7 +75531,7 @@
       </c>
       <c r="B1212" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1212" s="2" t="inlineStr">
@@ -76771,7 +76771,7 @@
       </c>
       <c r="B1232" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1232" s="2" t="inlineStr">
@@ -78135,7 +78135,7 @@
       </c>
       <c r="B1254" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1254" s="2" t="inlineStr">
@@ -78197,7 +78197,7 @@
       </c>
       <c r="B1255" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1255" s="2" t="inlineStr">
@@ -78259,7 +78259,7 @@
       </c>
       <c r="B1256" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1256" s="2" t="inlineStr">
@@ -78321,7 +78321,7 @@
       </c>
       <c r="B1257" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1257" s="2" t="inlineStr">
@@ -79623,7 +79623,7 @@
       </c>
       <c r="B1278" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1278" s="2" t="inlineStr">
@@ -80305,7 +80305,7 @@
       </c>
       <c r="B1289" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1289" s="2" t="inlineStr">
@@ -80367,7 +80367,7 @@
       </c>
       <c r="B1290" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1290" s="2" t="inlineStr">
@@ -80429,7 +80429,7 @@
       </c>
       <c r="B1291" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1291" s="2" t="inlineStr">
@@ -80615,7 +80615,7 @@
       </c>
       <c r="B1294" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1294" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -84955,7 +84955,7 @@
       </c>
       <c r="B1364" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1364" s="2" t="inlineStr">
@@ -85141,7 +85141,7 @@
       </c>
       <c r="B1367" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1367" s="2" t="inlineStr">
@@ -85265,7 +85265,7 @@
       </c>
       <c r="B1369" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1369" s="2" t="inlineStr">
@@ -85575,7 +85575,7 @@
       </c>
       <c r="B1374" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1374" s="2" t="inlineStr">
@@ -85637,7 +85637,7 @@
       </c>
       <c r="B1375" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1375" s="2" t="inlineStr">
@@ -85699,7 +85699,7 @@
       </c>
       <c r="B1376" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1376" s="2" t="inlineStr">
@@ -87497,7 +87497,7 @@
       </c>
       <c r="B1405" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1405" s="2" t="inlineStr">
@@ -88799,7 +88799,7 @@
       </c>
       <c r="B1426" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1426" s="2" t="inlineStr">
@@ -89171,7 +89171,7 @@
       </c>
       <c r="B1432" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1432" s="2" t="inlineStr">
@@ -89233,7 +89233,7 @@
       </c>
       <c r="B1433" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1433" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -91341,7 +91341,7 @@
       </c>
       <c r="B1467" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1467" s="2" t="inlineStr">
@@ -92023,7 +92023,7 @@
       </c>
       <c r="B1478" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1478" s="2" t="inlineStr">
@@ -92953,7 +92953,7 @@
       </c>
       <c r="B1493" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1493" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-13 02:20:51
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -7579,7 +7579,7 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
@@ -9191,7 +9191,7 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
@@ -22707,7 +22707,7 @@
       </c>
       <c r="B360" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C360" s="2" t="inlineStr">
@@ -34735,7 +34735,7 @@
       </c>
       <c r="B554" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C554" s="2" t="inlineStr">
@@ -35231,7 +35231,7 @@
       </c>
       <c r="B562" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C562" s="2" t="inlineStr">
@@ -38641,7 +38641,7 @@
       </c>
       <c r="B617" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C617" s="2" t="inlineStr">
@@ -40625,7 +40625,7 @@
       </c>
       <c r="B649" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C649" s="2" t="inlineStr">
@@ -43105,7 +43105,7 @@
       </c>
       <c r="B689" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C689" s="2" t="inlineStr">
@@ -43291,7 +43291,7 @@
       </c>
       <c r="B692" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C692" s="2" t="inlineStr">
@@ -49243,7 +49243,7 @@
       </c>
       <c r="B788" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C788" s="2" t="inlineStr">
@@ -52033,7 +52033,7 @@
       </c>
       <c r="B833" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C833" s="2" t="inlineStr">
@@ -58481,7 +58481,7 @@
       </c>
       <c r="B937" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C937" s="2" t="inlineStr">
@@ -58543,7 +58543,7 @@
       </c>
       <c r="B938" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C938" s="2" t="inlineStr">
@@ -60651,7 +60651,7 @@
       </c>
       <c r="B972" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C972" s="2" t="inlineStr">
@@ -61023,7 +61023,7 @@
       </c>
       <c r="B978" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C978" s="2" t="inlineStr">
@@ -63627,7 +63627,7 @@
       </c>
       <c r="B1020" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C1020" s="2" t="inlineStr">
@@ -70199,7 +70199,7 @@
       </c>
       <c r="B1126" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1126" s="2" t="inlineStr">
@@ -70261,7 +70261,7 @@
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
@@ -72121,7 +72121,7 @@
       </c>
       <c r="B1157" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1157" s="2" t="inlineStr">
@@ -72245,7 +72245,7 @@
       </c>
       <c r="B1159" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1159" s="2" t="inlineStr">
@@ -75221,7 +75221,7 @@
       </c>
       <c r="B1207" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1207" s="2" t="inlineStr">
@@ -75345,7 +75345,7 @@
       </c>
       <c r="B1209" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1209" s="2" t="inlineStr">
@@ -75593,7 +75593,7 @@
       </c>
       <c r="B1213" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1213" s="2" t="inlineStr">
@@ -76771,7 +76771,7 @@
       </c>
       <c r="B1232" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1232" s="2" t="inlineStr">
@@ -78135,7 +78135,7 @@
       </c>
       <c r="B1254" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1254" s="2" t="inlineStr">
@@ -78197,7 +78197,7 @@
       </c>
       <c r="B1255" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1255" s="2" t="inlineStr">
@@ -78321,7 +78321,7 @@
       </c>
       <c r="B1257" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1257" s="2" t="inlineStr">
@@ -79127,7 +79127,7 @@
       </c>
       <c r="B1270" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C1270" s="2" t="inlineStr">
@@ -80119,7 +80119,7 @@
       </c>
       <c r="B1286" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1286" s="2" t="inlineStr">
@@ -80367,7 +80367,7 @@
       </c>
       <c r="B1290" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1290" s="2" t="inlineStr">
@@ -84459,7 +84459,7 @@
       </c>
       <c r="B1356" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1356" s="2" t="inlineStr">
@@ -84521,7 +84521,7 @@
       </c>
       <c r="B1357" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1357" s="2" t="inlineStr">
@@ -84831,7 +84831,7 @@
       </c>
       <c r="B1362" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1362" s="2" t="inlineStr">
@@ -84955,7 +84955,7 @@
       </c>
       <c r="B1364" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1364" s="2" t="inlineStr">
@@ -85699,7 +85699,7 @@
       </c>
       <c r="B1376" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1376" s="2" t="inlineStr">
@@ -85761,7 +85761,7 @@
       </c>
       <c r="B1377" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1377" s="2" t="inlineStr">
@@ -87497,7 +87497,7 @@
       </c>
       <c r="B1405" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1405" s="2" t="inlineStr">
@@ -88861,7 +88861,7 @@
       </c>
       <c r="B1427" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1427" s="2" t="inlineStr">
@@ -89481,7 +89481,7 @@
       </c>
       <c r="B1437" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1437" s="2" t="inlineStr">
@@ -91217,7 +91217,7 @@
       </c>
       <c r="B1465" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1465" s="2" t="inlineStr">
@@ -91279,7 +91279,7 @@
       </c>
       <c r="B1466" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1466" s="2" t="inlineStr">
@@ -91341,7 +91341,7 @@
       </c>
       <c r="B1467" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1467" s="2" t="inlineStr">
@@ -92271,7 +92271,7 @@
       </c>
       <c r="B1482" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1482" s="2" t="inlineStr">
@@ -93635,7 +93635,7 @@
       </c>
       <c r="B1504" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1504" s="2" t="inlineStr">
@@ -93697,7 +93697,7 @@
       </c>
       <c r="B1505" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1505" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-13 02:40:50
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixa_42l.xlsx
+++ b/relatorio_analitico_caixa_42l.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -8757,7 +8757,7 @@
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
@@ -9191,7 +9191,7 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
@@ -15453,7 +15453,7 @@
       </c>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C243" s="2" t="inlineStr">
@@ -22707,7 +22707,7 @@
       </c>
       <c r="B360" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C360" s="2" t="inlineStr">
@@ -28659,7 +28659,7 @@
       </c>
       <c r="B456" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C456" s="2" t="inlineStr">
@@ -32131,7 +32131,7 @@
       </c>
       <c r="B512" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C512" s="2" t="inlineStr">
@@ -33495,7 +33495,7 @@
       </c>
       <c r="B534" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C534" s="2" t="inlineStr">
@@ -40625,7 +40625,7 @@
       </c>
       <c r="B649" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C649" s="2" t="inlineStr">
@@ -43043,7 +43043,7 @@
       </c>
       <c r="B688" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C688" s="2" t="inlineStr">
@@ -43105,7 +43105,7 @@
       </c>
       <c r="B689" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="C689" s="2" t="inlineStr">
@@ -44097,7 +44097,7 @@
       </c>
       <c r="B705" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C705" s="2" t="inlineStr">
@@ -44717,7 +44717,7 @@
       </c>
       <c r="B715" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C715" s="2" t="inlineStr">
@@ -47755,7 +47755,7 @@
       </c>
       <c r="B764" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C764" s="2" t="inlineStr">
@@ -51351,7 +51351,7 @@
       </c>
       <c r="B822" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C822" s="2" t="inlineStr">
@@ -51723,7 +51723,7 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C828" s="2" t="inlineStr">
@@ -51847,7 +51847,7 @@
       </c>
       <c r="B830" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C830" s="2" t="inlineStr">
@@ -51909,7 +51909,7 @@
       </c>
       <c r="B831" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C831" s="2" t="inlineStr">
@@ -51971,7 +51971,7 @@
       </c>
       <c r="B832" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C832" s="2" t="inlineStr">
@@ -52033,7 +52033,7 @@
       </c>
       <c r="B833" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C833" s="2" t="inlineStr">
@@ -54203,7 +54203,7 @@
       </c>
       <c r="B868" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="C868" s="2" t="inlineStr">
@@ -58605,7 +58605,7 @@
       </c>
       <c r="B939" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C939" s="2" t="inlineStr">
@@ -58667,7 +58667,7 @@
       </c>
       <c r="B940" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C940" s="2" t="inlineStr">
@@ -60713,7 +60713,7 @@
       </c>
       <c r="B973" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C973" s="2" t="inlineStr">
@@ -60775,7 +60775,7 @@
       </c>
       <c r="B974" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C974" s="2" t="inlineStr">
@@ -61147,7 +61147,7 @@
       </c>
       <c r="B980" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C980" s="2" t="inlineStr">
@@ -63751,7 +63751,7 @@
       </c>
       <c r="B1022" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1022" s="2" t="inlineStr">
@@ -70075,7 +70075,7 @@
       </c>
       <c r="B1124" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1124" s="2" t="inlineStr">
@@ -70385,7 +70385,7 @@
       </c>
       <c r="B1129" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1129" s="2" t="inlineStr">
@@ -72369,7 +72369,7 @@
       </c>
       <c r="B1161" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1161" s="2" t="inlineStr">
@@ -75283,7 +75283,7 @@
       </c>
       <c r="B1208" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1208" s="2" t="inlineStr">
@@ -75407,7 +75407,7 @@
       </c>
       <c r="B1210" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1210" s="2" t="inlineStr">
@@ -75717,7 +75717,7 @@
       </c>
       <c r="B1215" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1215" s="2" t="inlineStr">
@@ -76895,7 +76895,7 @@
       </c>
       <c r="B1234" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1234" s="2" t="inlineStr">
@@ -78321,7 +78321,7 @@
       </c>
       <c r="B1257" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1257" s="2" t="inlineStr">
@@ -78383,7 +78383,7 @@
       </c>
       <c r="B1258" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1258" s="2" t="inlineStr">
@@ -80243,7 +80243,7 @@
       </c>
       <c r="B1288" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1288" s="2" t="inlineStr">
@@ -80429,7 +80429,7 @@
       </c>
       <c r="B1291" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1291" s="2" t="inlineStr">
@@ -80553,7 +80553,7 @@
       </c>
       <c r="B1293" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1293" s="2" t="inlineStr">
@@ -84583,7 +84583,7 @@
       </c>
       <c r="B1358" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1358" s="2" t="inlineStr">
@@ -84645,7 +84645,7 @@
       </c>
       <c r="B1359" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1359" s="2" t="inlineStr">
@@ -84955,7 +84955,7 @@
       </c>
       <c r="B1364" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1364" s="2" t="inlineStr">
@@ -85389,7 +85389,7 @@
       </c>
       <c r="B1371" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1371" s="2" t="inlineStr">
@@ -85761,7 +85761,7 @@
       </c>
       <c r="B1377" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1377" s="2" t="inlineStr">
@@ -85823,7 +85823,7 @@
       </c>
       <c r="B1378" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1378" s="2" t="inlineStr">
@@ -89295,7 +89295,7 @@
       </c>
       <c r="B1434" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1434" s="2" t="inlineStr">
@@ -89357,7 +89357,7 @@
       </c>
       <c r="B1435" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="C1435" s="2" t="inlineStr">
@@ -91403,7 +91403,7 @@
       </c>
       <c r="B1468" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1468" s="2" t="inlineStr">
@@ -92147,7 +92147,7 @@
       </c>
       <c r="B1480" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="C1480" s="2" t="inlineStr">
@@ -93821,7 +93821,7 @@
       </c>
       <c r="B1507" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="C1507" s="2" t="inlineStr">

</xml_diff>